<commit_message>
Apply 7/25 costs to Shopify and regenerate report
- Update 116 ACTIVE variants' unitCost in Shopify to the 7/25 CJ costs
  (17 products down, none up); verified all 183 against the workbook
- Refresh the SKILL.md cost table with the new values and breakeven MERs
- Regenerate the 2026-07-25 report on the new cost basis

COGS drops 20,608 JPY over 7 days and 120,943 JPY over 30 days;
profit rises by the same amount. UV歯ブラシ and ワンピース move closer to
breakeven but stay negative, so no judgment flips.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017JNTxDUfjQsrckfss7YKHj
</commit_message>
<xml_diff>
--- a/data/reports/report-2026-07-25.xlsx
+++ b/data/reports/report-2026-07-25.xlsx
@@ -509,7 +509,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>LOOTY 日次損益レポート 2026-07-25定例（昨日=7/24 金実績・新原価・手数料3.49%）</t>
+          <t>LOOTY 日次損益レポート 2026-07-25定例（昨日=7/24 金実績・**7/25版新原価反映**・手数料3.49%）</t>
         </is>
       </c>
     </row>
@@ -591,21 +591,21 @@
         </is>
       </c>
       <c r="B6" s="4" t="n">
-        <v>398025</v>
+        <v>394927</v>
       </c>
       <c r="C6" s="4" t="inlineStr"/>
       <c r="D6" s="4" t="n">
-        <v>457475</v>
+        <v>454753</v>
       </c>
       <c r="E6" s="4" t="n">
-        <v>442013</v>
+        <v>439069</v>
       </c>
       <c r="F6" s="4" t="n">
-        <v>373652</v>
+        <v>369621</v>
       </c>
       <c r="G6" s="4" t="inlineStr">
         <is>
-          <t>-10%</t>
+          <t>-10.1%</t>
         </is>
       </c>
     </row>
@@ -641,21 +641,21 @@
         </is>
       </c>
       <c r="B8" s="4" t="n">
-        <v>374672</v>
+        <v>377770</v>
       </c>
       <c r="C8" s="4" t="inlineStr"/>
       <c r="D8" s="4" t="n">
-        <v>492437</v>
+        <v>495159</v>
       </c>
       <c r="E8" s="4" t="n">
-        <v>454035</v>
+        <v>456979</v>
       </c>
       <c r="F8" s="4" t="n">
-        <v>440685</v>
+        <v>444716</v>
       </c>
       <c r="G8" s="4" t="inlineStr">
         <is>
-          <t>-17.5% 🟡</t>
+          <t>-17.3% 🟡</t>
         </is>
       </c>
     </row>
@@ -667,28 +667,28 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>28.4%</t>
+          <t>28.6%</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr"/>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>32.9%</t>
+          <t>33.1%</t>
         </is>
       </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
-          <t>31.7%</t>
+          <t>31.9%</t>
         </is>
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>34.6%</t>
+          <t>34.9%</t>
         </is>
       </c>
       <c r="G9" s="4" t="inlineStr">
         <is>
-          <t>-3.3pt 🟡広告費比率上昇</t>
+          <t>-3.2pt 🟡広告費比率上昇</t>
         </is>
       </c>
     </row>
@@ -699,21 +699,21 @@
         </is>
       </c>
       <c r="B10" s="4" t="n">
-        <v>328625</v>
+        <v>331723</v>
       </c>
       <c r="C10" s="4" t="inlineStr"/>
       <c r="D10" s="4" t="n">
-        <v>440162</v>
+        <v>442884</v>
       </c>
       <c r="E10" s="4" t="n">
-        <v>403989</v>
+        <v>406933</v>
       </c>
       <c r="F10" s="4" t="n">
-        <v>396260</v>
+        <v>400291</v>
       </c>
       <c r="G10" s="4" t="inlineStr">
         <is>
-          <t>-18.7%</t>
+          <t>-18.5%</t>
         </is>
       </c>
     </row>
@@ -781,25 +781,25 @@
         <v>1319392</v>
       </c>
       <c r="C14" s="5" t="n">
-        <v>398025</v>
+        <v>394927</v>
       </c>
       <c r="D14" s="5" t="n">
         <v>546695</v>
       </c>
       <c r="E14" s="5" t="n">
-        <v>374672</v>
+        <v>377770</v>
       </c>
       <c r="F14" s="6" t="n">
-        <v>0.284</v>
+        <v>0.286</v>
       </c>
       <c r="G14" s="5" t="n">
         <v>46047</v>
       </c>
       <c r="H14" s="5" t="n">
-        <v>328625</v>
+        <v>331723</v>
       </c>
       <c r="I14" s="6" t="n">
-        <v>0.249</v>
+        <v>0.251</v>
       </c>
     </row>
     <row r="15">
@@ -812,25 +812,25 @@
         <v>4493555</v>
       </c>
       <c r="C15" s="5" t="n">
-        <v>1372426</v>
+        <v>1364261</v>
       </c>
       <c r="D15" s="5" t="n">
         <v>1643819</v>
       </c>
       <c r="E15" s="5" t="n">
-        <v>1477310</v>
+        <v>1485475</v>
       </c>
       <c r="F15" s="6" t="n">
-        <v>0.329</v>
+        <v>0.331</v>
       </c>
       <c r="G15" s="5" t="n">
         <v>156825</v>
       </c>
       <c r="H15" s="5" t="n">
-        <v>1320485</v>
+        <v>1328650</v>
       </c>
       <c r="I15" s="6" t="n">
-        <v>0.294</v>
+        <v>0.296</v>
       </c>
     </row>
     <row r="16">
@@ -843,25 +843,25 @@
         <v>10037916</v>
       </c>
       <c r="C16" s="5" t="n">
-        <v>3094089</v>
+        <v>3073481</v>
       </c>
       <c r="D16" s="5" t="n">
         <v>3765582</v>
       </c>
       <c r="E16" s="5" t="n">
-        <v>3178245</v>
+        <v>3198853</v>
       </c>
       <c r="F16" s="6" t="n">
-        <v>0.317</v>
+        <v>0.319</v>
       </c>
       <c r="G16" s="5" t="n">
         <v>350323</v>
       </c>
       <c r="H16" s="5" t="n">
-        <v>2827922</v>
+        <v>2848530</v>
       </c>
       <c r="I16" s="6" t="n">
-        <v>0.282</v>
+        <v>0.284</v>
       </c>
     </row>
     <row r="17">
@@ -874,25 +874,25 @@
         <v>38205301</v>
       </c>
       <c r="C17" s="5" t="n">
-        <v>11209574</v>
+        <v>11088631</v>
       </c>
       <c r="D17" s="5" t="n">
         <v>13775163</v>
       </c>
       <c r="E17" s="5" t="n">
-        <v>13220564</v>
+        <v>13341507</v>
       </c>
       <c r="F17" s="6" t="n">
-        <v>0.346</v>
+        <v>0.349</v>
       </c>
       <c r="G17" s="5" t="n">
         <v>1333365</v>
       </c>
       <c r="H17" s="5" t="n">
-        <v>11887199</v>
+        <v>12008142</v>
       </c>
       <c r="I17" s="6" t="n">
-        <v>0.311</v>
+        <v>0.314</v>
       </c>
     </row>
     <row r="18">
@@ -905,25 +905,25 @@
         <v>10037916</v>
       </c>
       <c r="C18" s="5" t="n">
-        <v>3094089</v>
+        <v>3073481</v>
       </c>
       <c r="D18" s="5" t="n">
         <v>3765582</v>
       </c>
       <c r="E18" s="5" t="n">
-        <v>3178245</v>
+        <v>3198853</v>
       </c>
       <c r="F18" s="6" t="n">
-        <v>0.317</v>
+        <v>0.319</v>
       </c>
       <c r="G18" s="5" t="n">
         <v>350323</v>
       </c>
       <c r="H18" s="5" t="n">
-        <v>2827922</v>
+        <v>2848530</v>
       </c>
       <c r="I18" s="6" t="n">
-        <v>0.282</v>
+        <v>0.284</v>
       </c>
     </row>
     <row r="20">
@@ -936,21 +936,21 @@
     <row r="21">
       <c r="A21" s="7" t="inlineStr">
         <is>
-          <t>・原価は2026-07-22更新のCJ最新原価。手数料ブレンド率3.49%（Shopify外部決済0.6%を実測反映）</t>
+          <t>・★原価は2026-07-25にCJ最新原価表でShopify全183バリエーションを一括更新（17商品値下げ・値上げゼロ）。手数料ブレンド率3.49%</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="7" t="inlineStr">
         <is>
-          <t>・現日予算はセット合算: 形状記憶60k(本体35k+テスト25k)、害虫73k(本体61k+テスト12k)、ナノガラス60k(本体50k+BC検証10k)、ディスペンサー12k(類似6k+全開放6k)</t>
+          <t>・新原価による原価減: 前日3,098円 / 3日8,165円 / 7日20,608円 / 30日120,943円（同額だけ利益が増加）</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="7" t="inlineStr">
         <is>
-          <t>・7日売上が1,003万で連日1,000万台維持。7/18累積=ちょうど7日窓と一致</t>
+          <t>・現日予算はセット合算: 形状記憶60k(本体35k+テスト25k)、害虫73k(本体61k+テスト12k)、ナノガラス60k(本体50k+BC検証10k)、ディスペンサー12k(類似6k+全開放6k)</t>
         </is>
       </c>
     </row>
@@ -965,7 +965,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P26"/>
+  <dimension ref="A1:P28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -1164,7 +1164,7 @@
         <v>1.28</v>
       </c>
       <c r="M3" s="13" t="n">
-        <v>1.55</v>
+        <v>1.54</v>
       </c>
       <c r="N3" s="11" t="n">
         <v>73000</v>
@@ -1220,7 +1220,7 @@
         <v>1.36</v>
       </c>
       <c r="M4" s="9" t="n">
-        <v>1.93</v>
+        <v>1.92</v>
       </c>
       <c r="N4" s="5" t="n">
         <v>60000</v>
@@ -1276,7 +1276,7 @@
         <v>1.23</v>
       </c>
       <c r="M5" s="13" t="n">
-        <v>1.22</v>
+        <v>1.23</v>
       </c>
       <c r="N5" s="11" t="n">
         <v>60000</v>
@@ -1444,7 +1444,7 @@
         <v>1.57</v>
       </c>
       <c r="M8" s="9" t="n">
-        <v>1.91</v>
+        <v>1.9</v>
       </c>
       <c r="N8" s="5" t="n">
         <v>34000</v>
@@ -1526,37 +1526,37 @@
         <v>321680</v>
       </c>
       <c r="C10" s="5" t="n">
-        <v>79137</v>
+        <v>72333</v>
       </c>
       <c r="D10" s="5" t="n">
         <v>154169</v>
       </c>
       <c r="E10" s="5" t="n">
-        <v>88374</v>
+        <v>95178</v>
       </c>
       <c r="F10" s="5" t="n">
         <v>43780</v>
       </c>
       <c r="G10" s="5" t="n">
-        <v>12628</v>
-      </c>
-      <c r="H10" s="8" t="n">
-        <v>0.288</v>
+        <v>13552</v>
+      </c>
+      <c r="H10" s="6" t="n">
+        <v>0.31</v>
       </c>
       <c r="I10" s="5" t="n">
-        <v>26173</v>
+        <v>28693</v>
       </c>
       <c r="J10" s="5" t="n">
-        <v>543288</v>
+        <v>576804</v>
       </c>
       <c r="K10" s="9" t="n">
         <v>2.09</v>
       </c>
       <c r="L10" s="9" t="n">
-        <v>1.33</v>
+        <v>1.29</v>
       </c>
       <c r="M10" s="9" t="n">
-        <v>0.76</v>
+        <v>0.8</v>
       </c>
       <c r="N10" s="5" t="n">
         <v>22000</v>
@@ -1582,37 +1582,37 @@
         <v>316940</v>
       </c>
       <c r="C11" s="11" t="n">
-        <v>132500</v>
+        <v>131705</v>
       </c>
       <c r="D11" s="11" t="n">
         <v>96961</v>
       </c>
       <c r="E11" s="11" t="n">
-        <v>87479</v>
+        <v>88274</v>
       </c>
       <c r="F11" s="11" t="n">
         <v>11960</v>
       </c>
       <c r="G11" s="14" t="n">
-        <v>-8854</v>
+        <v>-8824</v>
       </c>
       <c r="H11" s="8" t="n">
-        <v>-0.74</v>
+        <v>-0.738</v>
       </c>
       <c r="I11" s="11" t="n">
-        <v>35487</v>
+        <v>35832</v>
       </c>
       <c r="J11" s="11" t="n">
-        <v>236826</v>
+        <v>239361</v>
       </c>
       <c r="K11" s="13" t="n">
         <v>3.27</v>
       </c>
       <c r="L11" s="13" t="n">
-        <v>1.72</v>
+        <v>1.71</v>
       </c>
       <c r="M11" s="13" t="n">
-        <v>1.55</v>
+        <v>1.56</v>
       </c>
       <c r="N11" s="11" t="n">
         <v>16000</v>
@@ -1638,28 +1638,28 @@
         <v>238660</v>
       </c>
       <c r="C12" s="5" t="n">
-        <v>48000</v>
+        <v>47040</v>
       </c>
       <c r="D12" s="5" t="n">
         <v>119985</v>
       </c>
       <c r="E12" s="5" t="n">
-        <v>70675</v>
+        <v>71635</v>
       </c>
       <c r="F12" s="5" t="n">
         <v>31840</v>
       </c>
       <c r="G12" s="5" t="n">
-        <v>8214</v>
+        <v>8342</v>
       </c>
       <c r="H12" s="8" t="n">
-        <v>0.258</v>
+        <v>0.262</v>
       </c>
       <c r="I12" s="5" t="n">
-        <v>25355</v>
+        <v>25739</v>
       </c>
       <c r="J12" s="5" t="n">
-        <v>384920</v>
+        <v>389240</v>
       </c>
       <c r="K12" s="9" t="n">
         <v>1.99</v>
@@ -1687,51 +1687,51 @@
     <row r="13">
       <c r="A13" s="10" t="inlineStr">
         <is>
-          <t>健康サンダル</t>
+          <t>ムダ毛シェーバー</t>
         </is>
       </c>
       <c r="B13" s="11" t="n">
-        <v>178260</v>
+        <v>215280</v>
       </c>
       <c r="C13" s="11" t="n">
-        <v>44170</v>
+        <v>100728</v>
       </c>
       <c r="D13" s="11" t="n">
-        <v>91154</v>
+        <v>92441</v>
       </c>
       <c r="E13" s="11" t="n">
-        <v>42936</v>
+        <v>22111</v>
       </c>
       <c r="F13" s="11" t="n">
-        <v>24900</v>
+        <v>29900</v>
       </c>
       <c r="G13" s="11" t="n">
-        <v>5284</v>
+        <v>4611</v>
       </c>
       <c r="H13" s="8" t="n">
-        <v>0.212</v>
+        <v>0.154</v>
       </c>
       <c r="I13" s="11" t="n">
-        <v>25774</v>
+        <v>17139</v>
       </c>
       <c r="J13" s="11" t="n">
-        <v>302695</v>
+        <v>48109</v>
       </c>
       <c r="K13" s="13" t="n">
-        <v>1.96</v>
+        <v>2.33</v>
       </c>
       <c r="L13" s="13" t="n">
-        <v>1.33</v>
+        <v>1.88</v>
       </c>
       <c r="M13" s="13" t="n">
-        <v>0.63</v>
+        <v>0.45</v>
       </c>
       <c r="N13" s="11" t="n">
         <v>13000</v>
       </c>
       <c r="O13" s="10" t="inlineStr">
         <is>
-          <t>👀弱含み</t>
+          <t>✅黒字維持(7/27判定)</t>
         </is>
       </c>
       <c r="P13" s="10" t="inlineStr">
@@ -1743,389 +1743,425 @@
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t>優先配送</t>
+          <t>健康サンダル</t>
         </is>
       </c>
       <c r="B14" s="5" t="n">
-        <v>42880</v>
+        <v>178260</v>
       </c>
       <c r="C14" s="5" t="n">
-        <v>0</v>
+        <v>40670</v>
       </c>
       <c r="D14" s="5" t="n">
-        <v>0</v>
+        <v>91154</v>
       </c>
       <c r="E14" s="5" t="n">
-        <v>42880</v>
+        <v>46436</v>
       </c>
       <c r="F14" s="5" t="n">
-        <v>6432</v>
+        <v>24900</v>
       </c>
       <c r="G14" s="5" t="n">
-        <v>6432</v>
-      </c>
-      <c r="H14" s="6" t="n">
-        <v>1</v>
+        <v>5784</v>
+      </c>
+      <c r="H14" s="8" t="n">
+        <v>0.232</v>
       </c>
       <c r="I14" s="5" t="n">
-        <v>18224</v>
+        <v>27274</v>
       </c>
       <c r="J14" s="5" t="n">
-        <v>110952</v>
-      </c>
-      <c r="K14" s="4" t="inlineStr"/>
-      <c r="L14" s="4" t="inlineStr"/>
-      <c r="M14" s="4" t="inlineStr"/>
-      <c r="N14" s="4" t="inlineStr"/>
+        <v>320995</v>
+      </c>
+      <c r="K14" s="9" t="n">
+        <v>1.96</v>
+      </c>
+      <c r="L14" s="9" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="M14" s="9" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="N14" s="5" t="n">
+        <v>13000</v>
+      </c>
       <c r="O14" s="4" t="inlineStr">
         <is>
-          <t>📦広告なし</t>
+          <t>👀弱含み</t>
         </is>
       </c>
       <c r="P14" s="4" t="inlineStr">
         <is>
-          <t>−</t>
+          <t>13k維持</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="10" t="inlineStr">
         <is>
-          <t>瞬間冷却ハンディファン</t>
+          <t>瞬間冷感ポンチョ</t>
         </is>
       </c>
       <c r="B15" s="11" t="n">
-        <v>47840</v>
+        <v>159200</v>
       </c>
       <c r="C15" s="11" t="n">
-        <v>16952</v>
+        <v>39480</v>
       </c>
       <c r="D15" s="11" t="n">
-        <v>0</v>
+        <v>91828</v>
       </c>
       <c r="E15" s="11" t="n">
-        <v>30888</v>
+        <v>27892</v>
       </c>
       <c r="F15" s="11" t="n">
-        <v>5980</v>
+        <v>47760</v>
       </c>
       <c r="G15" s="11" t="n">
-        <v>3861</v>
+        <v>24112</v>
       </c>
       <c r="H15" s="12" t="n">
-        <v>0.646</v>
+        <v>0.505</v>
       </c>
       <c r="I15" s="11" t="n">
-        <v>19305</v>
+        <v>51827</v>
       </c>
       <c r="J15" s="11" t="n">
-        <v>69498</v>
-      </c>
-      <c r="K15" s="10" t="inlineStr"/>
-      <c r="L15" s="10" t="inlineStr"/>
-      <c r="M15" s="10" t="inlineStr"/>
-      <c r="N15" s="10" t="inlineStr"/>
+        <v>125094</v>
+      </c>
+      <c r="K15" s="13" t="n">
+        <v>1.73</v>
+      </c>
+      <c r="L15" s="13" t="n">
+        <v>1.33</v>
+      </c>
+      <c r="M15" s="13" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="N15" s="11" t="n">
+        <v>13000</v>
+      </c>
       <c r="O15" s="10" t="inlineStr">
         <is>
-          <t>📦広告なし</t>
+          <t>✅維持</t>
         </is>
       </c>
       <c r="P15" s="10" t="inlineStr">
         <is>
-          <t>−</t>
+          <t>13k維持</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t>瞬間冷感ポンチョ</t>
+          <t>携帯電動シェーバー</t>
         </is>
       </c>
       <c r="B16" s="5" t="n">
-        <v>159200</v>
+        <v>144420</v>
       </c>
       <c r="C16" s="5" t="n">
-        <v>40680</v>
+        <v>48804</v>
       </c>
       <c r="D16" s="5" t="n">
-        <v>91828</v>
+        <v>78644</v>
       </c>
       <c r="E16" s="5" t="n">
-        <v>26692</v>
+        <v>16972</v>
       </c>
       <c r="F16" s="5" t="n">
-        <v>47760</v>
-      </c>
-      <c r="G16" s="5" t="n">
-        <v>23752</v>
-      </c>
-      <c r="H16" s="6" t="n">
-        <v>0.497</v>
-      </c>
-      <c r="I16" s="5" t="n">
-        <v>50927</v>
+        <v>4980</v>
+      </c>
+      <c r="G16" s="15" t="n">
+        <v>-7092</v>
+      </c>
+      <c r="H16" s="8" t="n">
+        <v>-1.424</v>
+      </c>
+      <c r="I16" s="15" t="n">
+        <v>-652</v>
       </c>
       <c r="J16" s="5" t="n">
-        <v>122094</v>
+        <v>220759</v>
       </c>
       <c r="K16" s="9" t="n">
-        <v>1.73</v>
+        <v>1.84</v>
       </c>
       <c r="L16" s="9" t="n">
-        <v>1.34</v>
+        <v>1.51</v>
       </c>
       <c r="M16" s="9" t="n">
-        <v>0.39</v>
+        <v>0.33</v>
       </c>
       <c r="N16" s="5" t="n">
-        <v>13000</v>
+        <v>11000</v>
       </c>
       <c r="O16" s="4" t="inlineStr">
         <is>
-          <t>✅維持</t>
+          <t>👀前日弱</t>
         </is>
       </c>
       <c r="P16" s="4" t="inlineStr">
         <is>
-          <t>13k維持</t>
+          <t>11k維持</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="10" t="inlineStr">
         <is>
-          <t>ムダ毛シェーバー</t>
+          <t>UV歯ブラシ除菌器</t>
         </is>
       </c>
       <c r="B17" s="11" t="n">
-        <v>215280</v>
+        <v>125720</v>
       </c>
       <c r="C17" s="11" t="n">
-        <v>100728</v>
+        <v>45360</v>
       </c>
       <c r="D17" s="11" t="n">
-        <v>92441</v>
-      </c>
-      <c r="E17" s="11" t="n">
-        <v>22111</v>
+        <v>85489</v>
+      </c>
+      <c r="E17" s="14" t="n">
+        <v>-5129</v>
       </c>
       <c r="F17" s="11" t="n">
-        <v>29900</v>
+        <v>35920</v>
       </c>
       <c r="G17" s="11" t="n">
-        <v>4611</v>
-      </c>
-      <c r="H17" s="8" t="n">
-        <v>0.154</v>
+        <v>13193</v>
+      </c>
+      <c r="H17" s="12" t="n">
+        <v>0.367</v>
       </c>
       <c r="I17" s="11" t="n">
-        <v>17139</v>
+        <v>1425</v>
       </c>
       <c r="J17" s="11" t="n">
-        <v>48109</v>
+        <v>267661</v>
       </c>
       <c r="K17" s="13" t="n">
-        <v>2.33</v>
+        <v>1.47</v>
       </c>
       <c r="L17" s="13" t="n">
-        <v>1.88</v>
+        <v>1.56</v>
       </c>
       <c r="M17" s="13" t="n">
-        <v>0.45</v>
+        <v>-0.09</v>
       </c>
       <c r="N17" s="11" t="n">
-        <v>13000</v>
+        <v>10000</v>
       </c>
       <c r="O17" s="10" t="inlineStr">
         <is>
-          <t>✅黒字維持(7/27判定)</t>
+          <t>🔧複製リセット中(7/30)</t>
         </is>
       </c>
       <c r="P17" s="10" t="inlineStr">
         <is>
-          <t>13k維持</t>
+          <t>10k維持</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
         <is>
-          <t>携帯電動シェーバー</t>
+          <t>壁掛けディスペンサー</t>
         </is>
       </c>
       <c r="B18" s="5" t="n">
-        <v>144420</v>
+        <v>100700</v>
       </c>
       <c r="C18" s="5" t="n">
-        <v>49840</v>
+        <v>35732</v>
       </c>
       <c r="D18" s="5" t="n">
-        <v>78644</v>
-      </c>
-      <c r="E18" s="5" t="n">
-        <v>15936</v>
+        <v>94262</v>
+      </c>
+      <c r="E18" s="15" t="n">
+        <v>-29294</v>
       </c>
       <c r="F18" s="5" t="n">
-        <v>4980</v>
+        <v>12960</v>
       </c>
       <c r="G18" s="15" t="n">
-        <v>-7129</v>
+        <v>-2390</v>
       </c>
       <c r="H18" s="8" t="n">
-        <v>-1.432</v>
+        <v>-0.184</v>
       </c>
       <c r="I18" s="15" t="n">
-        <v>-948</v>
+        <v>-14004</v>
       </c>
       <c r="J18" s="5" t="n">
-        <v>213988</v>
+        <v>123009</v>
       </c>
       <c r="K18" s="9" t="n">
-        <v>1.84</v>
+        <v>1.07</v>
       </c>
       <c r="L18" s="9" t="n">
-        <v>1.53</v>
+        <v>1.55</v>
       </c>
       <c r="M18" s="9" t="n">
-        <v>0.31</v>
+        <v>-0.48</v>
       </c>
       <c r="N18" s="5" t="n">
-        <v>11000</v>
+        <v>12000</v>
       </c>
       <c r="O18" s="4" t="inlineStr">
         <is>
-          <t>👀前日弱</t>
+          <t>🚨全開放テスト中(8/6)</t>
         </is>
       </c>
       <c r="P18" s="4" t="inlineStr">
         <is>
-          <t>11k維持</t>
+          <t>6k+6k維持</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="10" t="inlineStr">
         <is>
-          <t>完全遮光・接触冷感UVハット</t>
+          <t>バランスケアスリッパ</t>
         </is>
       </c>
       <c r="B19" s="11" t="n">
-        <v>11960</v>
+        <v>84660</v>
       </c>
       <c r="C19" s="11" t="n">
-        <v>2870</v>
+        <v>22168</v>
       </c>
       <c r="D19" s="11" t="n">
-        <v>0</v>
+        <v>57798</v>
       </c>
       <c r="E19" s="11" t="n">
-        <v>9090</v>
+        <v>4694</v>
       </c>
       <c r="F19" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="G19" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="H19" s="10" t="inlineStr"/>
+        <v>4980</v>
+      </c>
+      <c r="G19" s="14" t="n">
+        <v>-1553</v>
+      </c>
+      <c r="H19" s="8" t="n">
+        <v>-0.312</v>
+      </c>
       <c r="I19" s="11" t="n">
-        <v>4545</v>
+        <v>8072</v>
       </c>
       <c r="J19" s="11" t="n">
-        <v>40905</v>
-      </c>
-      <c r="K19" s="10" t="inlineStr"/>
-      <c r="L19" s="10" t="inlineStr"/>
-      <c r="M19" s="10" t="inlineStr"/>
-      <c r="N19" s="10" t="inlineStr"/>
+        <v>94581</v>
+      </c>
+      <c r="K19" s="13" t="n">
+        <v>1.46</v>
+      </c>
+      <c r="L19" s="13" t="n">
+        <v>1.35</v>
+      </c>
+      <c r="M19" s="13" t="n">
+        <v>0.11</v>
+      </c>
+      <c r="N19" s="11" t="n">
+        <v>5000</v>
+      </c>
       <c r="O19" s="10" t="inlineStr">
         <is>
-          <t>📦広告なし</t>
+          <t>🔧CR効果判定は7/29</t>
         </is>
       </c>
       <c r="P19" s="10" t="inlineStr">
         <is>
-          <t>−</t>
+          <t>5k維持</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
         <is>
-          <t>ネックマッサージャー</t>
+          <t>湯上がりガーゼワンピース</t>
         </is>
       </c>
       <c r="B20" s="5" t="n">
-        <v>9980</v>
+        <v>80720</v>
       </c>
       <c r="C20" s="5" t="n">
-        <v>3136</v>
+        <v>27552</v>
       </c>
       <c r="D20" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="E20" s="5" t="n">
-        <v>6844</v>
+        <v>56119</v>
+      </c>
+      <c r="E20" s="15" t="n">
+        <v>-2951</v>
       </c>
       <c r="F20" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="G20" s="5" t="n">
-        <v>0</v>
+      <c r="G20" s="15" t="n">
+        <v>-6289</v>
       </c>
       <c r="H20" s="4" t="inlineStr"/>
-      <c r="I20" s="5" t="n">
-        <v>0</v>
+      <c r="I20" s="15" t="n">
+        <v>-6539</v>
       </c>
       <c r="J20" s="5" t="n">
-        <v>6844</v>
-      </c>
-      <c r="K20" s="4" t="inlineStr"/>
-      <c r="L20" s="4" t="inlineStr"/>
-      <c r="M20" s="4" t="inlineStr"/>
-      <c r="N20" s="4" t="inlineStr"/>
+        <v>108918</v>
+      </c>
+      <c r="K20" s="9" t="n">
+        <v>1.44</v>
+      </c>
+      <c r="L20" s="9" t="n">
+        <v>1.52</v>
+      </c>
+      <c r="M20" s="9" t="n">
+        <v>-0.08</v>
+      </c>
+      <c r="N20" s="5" t="n">
+        <v>6500</v>
+      </c>
       <c r="O20" s="4" t="inlineStr">
         <is>
-          <t>📦広告なし</t>
+          <t>🔧段階②判定は7/26</t>
         </is>
       </c>
       <c r="P20" s="4" t="inlineStr">
         <is>
-          <t>−</t>
+          <t>6.5k維持</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="10" t="inlineStr">
         <is>
-          <t>リカバリーサンダル</t>
+          <t>瞬間冷却ハンディファン</t>
         </is>
       </c>
       <c r="B21" s="11" t="n">
-        <v>7960</v>
+        <v>47840</v>
       </c>
       <c r="C21" s="11" t="n">
-        <v>2750</v>
+        <v>16424</v>
       </c>
       <c r="D21" s="11" t="n">
         <v>0</v>
       </c>
       <c r="E21" s="11" t="n">
-        <v>5210</v>
+        <v>31416</v>
       </c>
       <c r="F21" s="11" t="n">
-        <v>0</v>
+        <v>5980</v>
       </c>
       <c r="G21" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="H21" s="10" t="inlineStr"/>
+        <v>3927</v>
+      </c>
+      <c r="H21" s="12" t="n">
+        <v>0.657</v>
+      </c>
       <c r="I21" s="11" t="n">
-        <v>0</v>
+        <v>19635</v>
       </c>
       <c r="J21" s="11" t="n">
-        <v>18235</v>
+        <v>70686</v>
       </c>
       <c r="K21" s="10" t="inlineStr"/>
       <c r="L21" s="10" t="inlineStr"/>
@@ -2145,222 +2181,186 @@
     <row r="22">
       <c r="A22" s="4" t="inlineStr">
         <is>
-          <t>バランスケアスリッパ</t>
+          <t>優先配送</t>
         </is>
       </c>
       <c r="B22" s="5" t="n">
-        <v>84660</v>
+        <v>42880</v>
       </c>
       <c r="C22" s="5" t="n">
-        <v>22168</v>
+        <v>0</v>
       </c>
       <c r="D22" s="5" t="n">
-        <v>57798</v>
+        <v>0</v>
       </c>
       <c r="E22" s="5" t="n">
-        <v>4694</v>
+        <v>42880</v>
       </c>
       <c r="F22" s="5" t="n">
-        <v>4980</v>
-      </c>
-      <c r="G22" s="15" t="n">
-        <v>-1553</v>
-      </c>
-      <c r="H22" s="8" t="n">
-        <v>-0.312</v>
+        <v>6432</v>
+      </c>
+      <c r="G22" s="5" t="n">
+        <v>6432</v>
+      </c>
+      <c r="H22" s="6" t="n">
+        <v>1</v>
       </c>
       <c r="I22" s="5" t="n">
-        <v>8072</v>
+        <v>18224</v>
       </c>
       <c r="J22" s="5" t="n">
-        <v>94581</v>
-      </c>
-      <c r="K22" s="9" t="n">
-        <v>1.46</v>
-      </c>
-      <c r="L22" s="9" t="n">
-        <v>1.35</v>
-      </c>
-      <c r="M22" s="9" t="n">
-        <v>0.11</v>
-      </c>
-      <c r="N22" s="5" t="n">
-        <v>5000</v>
-      </c>
+        <v>110952</v>
+      </c>
+      <c r="K22" s="4" t="inlineStr"/>
+      <c r="L22" s="4" t="inlineStr"/>
+      <c r="M22" s="4" t="inlineStr"/>
+      <c r="N22" s="4" t="inlineStr"/>
       <c r="O22" s="4" t="inlineStr">
         <is>
-          <t>🔧CR効果判定は7/29</t>
+          <t>📦広告なし</t>
         </is>
       </c>
       <c r="P22" s="4" t="inlineStr">
         <is>
-          <t>5k維持</t>
+          <t>−</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="10" t="inlineStr">
         <is>
-          <t>湯上がりガーゼワンピース</t>
+          <t>完全遮光・接触冷感UVハット</t>
         </is>
       </c>
       <c r="B23" s="11" t="n">
-        <v>80720</v>
+        <v>11960</v>
       </c>
       <c r="C23" s="11" t="n">
-        <v>28672</v>
+        <v>2822</v>
       </c>
       <c r="D23" s="11" t="n">
-        <v>56119</v>
-      </c>
-      <c r="E23" s="14" t="n">
-        <v>-4071</v>
+        <v>0</v>
+      </c>
+      <c r="E23" s="11" t="n">
+        <v>9138</v>
       </c>
       <c r="F23" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="G23" s="14" t="n">
-        <v>-6289</v>
+      <c r="G23" s="11" t="n">
+        <v>0</v>
       </c>
       <c r="H23" s="10" t="inlineStr"/>
-      <c r="I23" s="14" t="n">
-        <v>-6779</v>
+      <c r="I23" s="11" t="n">
+        <v>4569</v>
       </c>
       <c r="J23" s="11" t="n">
-        <v>96918</v>
-      </c>
-      <c r="K23" s="13" t="n">
-        <v>1.44</v>
-      </c>
-      <c r="L23" s="13" t="n">
-        <v>1.55</v>
-      </c>
-      <c r="M23" s="13" t="n">
-        <v>-0.11</v>
-      </c>
-      <c r="N23" s="11" t="n">
-        <v>6500</v>
-      </c>
+        <v>41121</v>
+      </c>
+      <c r="K23" s="10" t="inlineStr"/>
+      <c r="L23" s="10" t="inlineStr"/>
+      <c r="M23" s="10" t="inlineStr"/>
+      <c r="N23" s="10" t="inlineStr"/>
       <c r="O23" s="10" t="inlineStr">
         <is>
-          <t>🔧段階②判定は7/26</t>
+          <t>📦広告なし</t>
         </is>
       </c>
       <c r="P23" s="10" t="inlineStr">
         <is>
-          <t>6.5k維持</t>
+          <t>−</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="4" t="inlineStr">
         <is>
-          <t>UV歯ブラシ除菌器</t>
+          <t>ネックマッサージャー</t>
         </is>
       </c>
       <c r="B24" s="5" t="n">
-        <v>125720</v>
+        <v>9980</v>
       </c>
       <c r="C24" s="5" t="n">
-        <v>48720</v>
+        <v>3034</v>
       </c>
       <c r="D24" s="5" t="n">
-        <v>85489</v>
-      </c>
-      <c r="E24" s="15" t="n">
-        <v>-8489</v>
+        <v>0</v>
+      </c>
+      <c r="E24" s="5" t="n">
+        <v>6946</v>
       </c>
       <c r="F24" s="5" t="n">
-        <v>35920</v>
+        <v>0</v>
       </c>
       <c r="G24" s="5" t="n">
-        <v>12233</v>
-      </c>
-      <c r="H24" s="6" t="n">
-        <v>0.341</v>
-      </c>
-      <c r="I24" s="15" t="n">
-        <v>-15</v>
+        <v>0</v>
+      </c>
+      <c r="H24" s="4" t="inlineStr"/>
+      <c r="I24" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="J24" s="5" t="n">
-        <v>241021</v>
-      </c>
-      <c r="K24" s="9" t="n">
-        <v>1.47</v>
-      </c>
-      <c r="L24" s="9" t="n">
-        <v>1.63</v>
-      </c>
-      <c r="M24" s="9" t="n">
-        <v>-0.16</v>
-      </c>
-      <c r="N24" s="5" t="n">
-        <v>10000</v>
-      </c>
+        <v>6946</v>
+      </c>
+      <c r="K24" s="4" t="inlineStr"/>
+      <c r="L24" s="4" t="inlineStr"/>
+      <c r="M24" s="4" t="inlineStr"/>
+      <c r="N24" s="4" t="inlineStr"/>
       <c r="O24" s="4" t="inlineStr">
         <is>
-          <t>🔧複製リセット中(7/30)</t>
+          <t>📦広告なし</t>
         </is>
       </c>
       <c r="P24" s="4" t="inlineStr">
         <is>
-          <t>10k維持</t>
+          <t>−</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="10" t="inlineStr">
         <is>
-          <t>壁掛けディスペンサー</t>
+          <t>リカバリーサンダル</t>
         </is>
       </c>
       <c r="B25" s="11" t="n">
-        <v>100700</v>
+        <v>7960</v>
       </c>
       <c r="C25" s="11" t="n">
-        <v>36755</v>
+        <v>2618</v>
       </c>
       <c r="D25" s="11" t="n">
-        <v>94262</v>
-      </c>
-      <c r="E25" s="14" t="n">
-        <v>-30317</v>
+        <v>0</v>
+      </c>
+      <c r="E25" s="11" t="n">
+        <v>5342</v>
       </c>
       <c r="F25" s="11" t="n">
-        <v>12960</v>
-      </c>
-      <c r="G25" s="14" t="n">
-        <v>-2483</v>
-      </c>
-      <c r="H25" s="8" t="n">
-        <v>-0.192</v>
-      </c>
-      <c r="I25" s="14" t="n">
-        <v>-14190</v>
+        <v>0</v>
+      </c>
+      <c r="G25" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H25" s="10" t="inlineStr"/>
+      <c r="I25" s="11" t="n">
+        <v>0</v>
       </c>
       <c r="J25" s="11" t="n">
-        <v>112314</v>
-      </c>
-      <c r="K25" s="13" t="n">
-        <v>1.07</v>
-      </c>
-      <c r="L25" s="13" t="n">
-        <v>1.57</v>
-      </c>
-      <c r="M25" s="13" t="n">
-        <v>-0.51</v>
-      </c>
-      <c r="N25" s="11" t="n">
-        <v>12000</v>
-      </c>
+        <v>18697</v>
+      </c>
+      <c r="K25" s="10" t="inlineStr"/>
+      <c r="L25" s="10" t="inlineStr"/>
+      <c r="M25" s="10" t="inlineStr"/>
+      <c r="N25" s="10" t="inlineStr"/>
       <c r="O25" s="10" t="inlineStr">
         <is>
-          <t>🚨全開放テスト中(8/6)</t>
+          <t>📦広告なし</t>
         </is>
       </c>
       <c r="P25" s="10" t="inlineStr">
         <is>
-          <t>6k+6k維持</t>
+          <t>−</t>
         </is>
       </c>
     </row>
@@ -2393,7 +2393,7 @@
         <v>0</v>
       </c>
       <c r="J26" s="5" t="n">
-        <v>55764</v>
+        <v>56700</v>
       </c>
       <c r="K26" s="4" t="inlineStr"/>
       <c r="L26" s="4" t="inlineStr"/>
@@ -2410,6 +2410,98 @@
         </is>
       </c>
     </row>
+    <row r="27">
+      <c r="A27" s="10" t="inlineStr">
+        <is>
+          <t>姿勢サポートベルト</t>
+        </is>
+      </c>
+      <c r="B27" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="C27" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="D27" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="E27" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="F27" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="G27" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H27" s="10" t="inlineStr"/>
+      <c r="I27" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="J27" s="11" t="n">
+        <v>4551</v>
+      </c>
+      <c r="K27" s="10" t="inlineStr"/>
+      <c r="L27" s="10" t="inlineStr"/>
+      <c r="M27" s="10" t="inlineStr"/>
+      <c r="N27" s="10" t="inlineStr"/>
+      <c r="O27" s="10" t="inlineStr">
+        <is>
+          <t>📦広告なし</t>
+        </is>
+      </c>
+      <c r="P27" s="10" t="inlineStr">
+        <is>
+          <t>−</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>癒しの指圧マット</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C28" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D28" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E28" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F28" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G28" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H28" s="4" t="inlineStr"/>
+      <c r="I28" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J28" s="5" t="n">
+        <v>4332</v>
+      </c>
+      <c r="K28" s="4" t="inlineStr"/>
+      <c r="L28" s="4" t="inlineStr"/>
+      <c r="M28" s="4" t="inlineStr"/>
+      <c r="N28" s="4" t="inlineStr"/>
+      <c r="O28" s="4" t="inlineStr">
+        <is>
+          <t>📦広告なし</t>
+        </is>
+      </c>
+      <c r="P28" s="4" t="inlineStr">
+        <is>
+          <t>−</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Decompose margin and give per-product actions across levers
Margin alone does not say what to fix, and a single day of it says
nothing at all for low-volume products. Add both halves:

- Product sheet gains 7日利益率 / 原価率 / 広告費率 and a 3日利益率 that
  only fills in for products selling 20+ units a day; cost ratio over 33%
  and ad ratio over 40% shade red so the bottleneck reads at a glance
- Section 7c: how 利益率 and MER relate, the volume threshold behind the
  3-day column, and the price-increase breakeven formula
- Section 7d:每 product now carries actions across ad, cost, price, AOV,
  landing page and season rather than a budget line alone

Measured over 5 days: 4WAY swings 6pt a day, 携帯電動シェーバー 64pt.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017JNTxDUfjQsrckfss7YKHj
</commit_message>
<xml_diff>
--- a/data/reports/report-2026-07-25.xlsx
+++ b/data/reports/report-2026-07-25.xlsx
@@ -73,6 +73,11 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="00FADBD8"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="00FFF2A8"/>
       </patternFill>
     </fill>
@@ -84,11 +89,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00F2F6FC"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FADBD8"/>
       </patternFill>
     </fill>
   </fills>
@@ -118,7 +118,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -130,15 +130,23 @@
     <xf numFmtId="164" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="4" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="4" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="2" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="2" fontId="4" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="4" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="4" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="2" fontId="4" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="2" fontId="4" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="3" fontId="4" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="4" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="2" fontId="4" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="2" fontId="4" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="2" fontId="4" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="3" fontId="6" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="6" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="6" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="6" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -505,7 +513,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I25"/>
+  <dimension ref="A1:I28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -981,6 +989,27 @@
         </is>
       </c>
     </row>
+    <row r="26">
+      <c r="A26" s="7" t="inlineStr">
+        <is>
+          <t>・★7日利益率 = 1 − 原価率 − 広告費率。MERとは 利益率 = 1 − 原価率 − 1/MER で対応する（同じ情報を別角度で見たもの）</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="7" t="inlineStr">
+        <is>
+          <t>・★3日利益率は日販20個以上の商品のみ表示。それ未満は日次のブレが大きく3日平均では実力を測れないため「−」</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="7" t="inlineStr">
+        <is>
+          <t>・★ボトルネック判定: 原価率&gt;33%（赤）→原価・価格で手当て / 広告費率&gt;40%（赤）→広告で手当て</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -992,29 +1021,33 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q28"/>
+  <dimension ref="A1:U28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
     <col width="11" customWidth="1" min="2" max="2"/>
-    <col width="11" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
     <col width="11" customWidth="1" min="4" max="4"/>
     <col width="11" customWidth="1" min="5" max="5"/>
-    <col width="10" customWidth="1" min="6" max="6"/>
-    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="9" customWidth="1" min="6" max="6"/>
+    <col width="8" customWidth="1" min="7" max="7"/>
     <col width="9" customWidth="1" min="8" max="8"/>
-    <col width="10" customWidth="1" min="9" max="9"/>
-    <col width="11" customWidth="1" min="10" max="10"/>
-    <col width="8" customWidth="1" min="11" max="11"/>
-    <col width="7" customWidth="1" min="12" max="12"/>
-    <col width="8" customWidth="1" min="13" max="13"/>
-    <col width="9" customWidth="1" min="14" max="14"/>
-    <col width="12" customWidth="1" min="15" max="15"/>
-    <col width="22" customWidth="1" min="16" max="16"/>
-    <col width="16" customWidth="1" min="17" max="17"/>
+    <col width="9" customWidth="1" min="9" max="9"/>
+    <col width="10" customWidth="1" min="10" max="10"/>
+    <col width="10" customWidth="1" min="11" max="11"/>
+    <col width="9" customWidth="1" min="12" max="12"/>
+    <col width="10" customWidth="1" min="13" max="13"/>
+    <col width="11" customWidth="1" min="14" max="14"/>
+    <col width="9" customWidth="1" min="15" max="15"/>
+    <col width="7" customWidth="1" min="16" max="16"/>
+    <col width="7" customWidth="1" min="17" max="17"/>
+    <col width="8" customWidth="1" min="18" max="18"/>
+    <col width="11" customWidth="1" min="19" max="19"/>
+    <col width="20" customWidth="1" min="20" max="20"/>
+    <col width="52" customWidth="1" min="21" max="21"/>
   </cols>
   <sheetData>
-    <row r="1" ht="28" customHeight="1">
+    <row r="1" ht="30" customHeight="1">
       <c r="A1" s="3" t="inlineStr">
         <is>
           <t>商品</t>
@@ -1042,62 +1075,82 @@
       </c>
       <c r="F1" s="3" t="inlineStr">
         <is>
+          <t>7日利益率</t>
+        </is>
+      </c>
+      <c r="G1" s="3" t="inlineStr">
+        <is>
+          <t>原価率</t>
+        </is>
+      </c>
+      <c r="H1" s="3" t="inlineStr">
+        <is>
+          <t>広告費率</t>
+        </is>
+      </c>
+      <c r="I1" s="3" t="inlineStr">
+        <is>
+          <t>3日利益率</t>
+        </is>
+      </c>
+      <c r="J1" s="3" t="inlineStr">
+        <is>
           <t>前日売上</t>
         </is>
       </c>
-      <c r="G1" s="3" t="inlineStr">
+      <c r="K1" s="3" t="inlineStr">
         <is>
           <t>前日利益</t>
         </is>
       </c>
-      <c r="H1" s="3" t="inlineStr">
+      <c r="L1" s="3" t="inlineStr">
         <is>
           <t>前日利益率</t>
         </is>
       </c>
-      <c r="I1" s="3" t="inlineStr">
+      <c r="M1" s="3" t="inlineStr">
         <is>
           <t>3日利益</t>
         </is>
       </c>
-      <c r="J1" s="3" t="inlineStr">
+      <c r="N1" s="3" t="inlineStr">
         <is>
           <t>30日利益</t>
         </is>
       </c>
-      <c r="K1" s="3" t="inlineStr">
+      <c r="O1" s="3" t="inlineStr">
         <is>
           <t>MER(7日)</t>
         </is>
       </c>
-      <c r="L1" s="3" t="inlineStr">
+      <c r="P1" s="3" t="inlineStr">
         <is>
           <t>分岐</t>
         </is>
       </c>
-      <c r="M1" s="3" t="inlineStr">
+      <c r="Q1" s="3" t="inlineStr">
         <is>
           <t>余裕</t>
         </is>
       </c>
-      <c r="N1" s="3" t="inlineStr">
+      <c r="R1" s="3" t="inlineStr">
         <is>
           <t>増分MER</t>
         </is>
       </c>
-      <c r="O1" s="3" t="inlineStr">
+      <c r="S1" s="3" t="inlineStr">
         <is>
           <t>現日予算(円)</t>
         </is>
       </c>
-      <c r="P1" s="3" t="inlineStr">
+      <c r="T1" s="3" t="inlineStr">
         <is>
           <t>判定</t>
         </is>
       </c>
-      <c r="Q1" s="3" t="inlineStr">
-        <is>
-          <t>予算提案</t>
+      <c r="U1" s="3" t="inlineStr">
+        <is>
+          <t>推奨アクション</t>
         </is>
       </c>
     </row>
@@ -1119,101 +1172,125 @@
       <c r="E2" s="5" t="n">
         <v>862663</v>
       </c>
-      <c r="F2" s="5" t="n">
+      <c r="F2" s="6" t="n">
+        <v>0.4001</v>
+      </c>
+      <c r="G2" s="8" t="n">
+        <v>0.3474</v>
+      </c>
+      <c r="H2" s="6" t="n">
+        <v>0.2526</v>
+      </c>
+      <c r="I2" s="6" t="n">
+        <v>0.3872</v>
+      </c>
+      <c r="J2" s="5" t="n">
         <v>219120</v>
       </c>
-      <c r="G2" s="5" t="n">
+      <c r="K2" s="5" t="n">
         <v>59860</v>
       </c>
-      <c r="H2" s="8" t="n">
+      <c r="L2" s="9" t="n">
         <v>0.273</v>
       </c>
-      <c r="I2" s="5" t="n">
+      <c r="M2" s="5" t="n">
         <v>364412</v>
       </c>
-      <c r="J2" s="5" t="n">
+      <c r="N2" s="5" t="n">
         <v>2574399</v>
       </c>
-      <c r="K2" s="9" t="n">
+      <c r="O2" s="10" t="n">
         <v>3.96</v>
       </c>
-      <c r="L2" s="9" t="n">
+      <c r="P2" s="10" t="n">
         <v>1.53</v>
       </c>
-      <c r="M2" s="9" t="n">
+      <c r="Q2" s="10" t="n">
         <v>2.43</v>
       </c>
-      <c r="N2" s="10" t="n">
+      <c r="R2" s="11" t="n">
         <v>3.34</v>
       </c>
-      <c r="O2" s="5" t="n">
+      <c r="S2" s="5" t="n">
         <v>85000</v>
       </c>
-      <c r="P2" s="4" t="inlineStr">
+      <c r="T2" s="4" t="inlineStr">
         <is>
           <t>✅増分3.34(7/28判定)</t>
         </is>
       </c>
-      <c r="Q2" s="4" t="inlineStr">
-        <is>
-          <t>85k据置</t>
+      <c r="U2" s="12" t="inlineStr">
+        <is>
+          <t>①予算95k据置→7/28に増分MER判定（≥2.91で110kへ）②原価率34.7%が唯一の弱点。CJに数量交渉（月1,300個の最大SKU＝交渉力あり）③+500円値上げは13.3%減までOK、8月中旬の需要減局面で試す価値あり</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="11" t="inlineStr">
+      <c r="A3" s="13" t="inlineStr">
         <is>
           <t>害虫ブロッカー</t>
         </is>
       </c>
-      <c r="B3" s="12" t="n">
+      <c r="B3" s="14" t="n">
         <v>1404940</v>
       </c>
-      <c r="C3" s="12" t="n">
+      <c r="C3" s="14" t="n">
         <v>303450</v>
       </c>
-      <c r="D3" s="12" t="n">
+      <c r="D3" s="14" t="n">
         <v>497927</v>
       </c>
-      <c r="E3" s="12" t="n">
+      <c r="E3" s="14" t="n">
         <v>603563</v>
       </c>
-      <c r="F3" s="12" t="n">
+      <c r="F3" s="15" t="n">
+        <v>0.4296</v>
+      </c>
+      <c r="G3" s="15" t="n">
+        <v>0.216</v>
+      </c>
+      <c r="H3" s="15" t="n">
+        <v>0.3544</v>
+      </c>
+      <c r="I3" s="15" t="n">
+        <v>0.4079</v>
+      </c>
+      <c r="J3" s="14" t="n">
         <v>222880</v>
       </c>
-      <c r="G3" s="12" t="n">
+      <c r="K3" s="14" t="n">
         <v>102560</v>
       </c>
-      <c r="H3" s="13" t="n">
+      <c r="L3" s="15" t="n">
         <v>0.46</v>
       </c>
-      <c r="I3" s="12" t="n">
+      <c r="M3" s="14" t="n">
         <v>235387</v>
       </c>
-      <c r="J3" s="12" t="n">
+      <c r="N3" s="14" t="n">
         <v>3975773</v>
       </c>
-      <c r="K3" s="14" t="n">
+      <c r="O3" s="16" t="n">
         <v>2.82</v>
       </c>
-      <c r="L3" s="14" t="n">
+      <c r="P3" s="16" t="n">
         <v>1.28</v>
       </c>
-      <c r="M3" s="14" t="n">
+      <c r="Q3" s="16" t="n">
         <v>1.54</v>
       </c>
-      <c r="N3" s="11" t="inlineStr"/>
-      <c r="O3" s="12" t="n">
+      <c r="R3" s="13" t="inlineStr"/>
+      <c r="S3" s="14" t="n">
         <v>73000</v>
       </c>
-      <c r="P3" s="11" t="inlineStr">
+      <c r="T3" s="13" t="inlineStr">
         <is>
           <t>✅維持</t>
         </is>
       </c>
-      <c r="Q3" s="11" t="inlineStr">
-        <is>
-          <t>73k維持</t>
+      <c r="U3" s="17" t="inlineStr">
+        <is>
+          <t>①MER2.82が目標2.91を僅かに下回る＝増額は率を薄める。据置が正解②原価率21.6%は最良でボトルネックなし③30日利益398万の最大の稼ぎ頭。触らないことが最大の打ち手④8月後半から需要減。9月に段階減額の計画を</t>
         </is>
       </c>
     </row>
@@ -1235,101 +1312,125 @@
       <c r="E4" s="5" t="n">
         <v>600921</v>
       </c>
-      <c r="F4" s="5" t="n">
+      <c r="F4" s="6" t="n">
+        <v>0.4325</v>
+      </c>
+      <c r="G4" s="6" t="n">
+        <v>0.2629</v>
+      </c>
+      <c r="H4" s="6" t="n">
+        <v>0.3047</v>
+      </c>
+      <c r="I4" s="6" t="n">
+        <v>0.468</v>
+      </c>
+      <c r="J4" s="5" t="n">
         <v>169320</v>
       </c>
-      <c r="G4" s="5" t="n">
+      <c r="K4" s="5" t="n">
         <v>67789</v>
       </c>
-      <c r="H4" s="6" t="n">
+      <c r="L4" s="6" t="n">
         <v>0.4</v>
       </c>
-      <c r="I4" s="5" t="n">
+      <c r="M4" s="5" t="n">
         <v>307648</v>
       </c>
-      <c r="J4" s="5" t="n">
+      <c r="N4" s="5" t="n">
         <v>2062030</v>
       </c>
-      <c r="K4" s="9" t="n">
+      <c r="O4" s="10" t="n">
         <v>3.28</v>
       </c>
-      <c r="L4" s="9" t="n">
+      <c r="P4" s="10" t="n">
         <v>1.36</v>
       </c>
-      <c r="M4" s="9" t="n">
+      <c r="Q4" s="10" t="n">
         <v>1.92</v>
       </c>
-      <c r="N4" s="4" t="inlineStr"/>
-      <c r="O4" s="5" t="n">
+      <c r="R4" s="4" t="inlineStr"/>
+      <c r="S4" s="5" t="n">
         <v>60000</v>
       </c>
-      <c r="P4" s="4" t="inlineStr">
+      <c r="T4" s="4" t="inlineStr">
         <is>
           <t>✅維持</t>
         </is>
       </c>
-      <c r="Q4" s="4" t="inlineStr">
-        <is>
-          <t>60k維持</t>
+      <c r="U4" s="12" t="inlineStr">
+        <is>
+          <t>①MER3.28・原価率26.3%とも健全。据置②完全遮光と同一SPUのため2本合算で判断（合算MER3.22）③日傘は8月お盆明けから急減。8/15を減額開始の目安に</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="11" t="inlineStr">
+      <c r="A5" s="13" t="inlineStr">
         <is>
           <t>ナノガラス脱毛パッド</t>
         </is>
       </c>
-      <c r="B5" s="12" t="n">
+      <c r="B5" s="14" t="n">
         <v>911720</v>
       </c>
-      <c r="C5" s="12" t="n">
+      <c r="C5" s="14" t="n">
         <v>172146</v>
       </c>
-      <c r="D5" s="12" t="n">
+      <c r="D5" s="14" t="n">
         <v>371009</v>
       </c>
-      <c r="E5" s="12" t="n">
+      <c r="E5" s="14" t="n">
         <v>368565</v>
       </c>
-      <c r="F5" s="12" t="n">
+      <c r="F5" s="15" t="n">
+        <v>0.4043</v>
+      </c>
+      <c r="G5" s="15" t="n">
+        <v>0.1888</v>
+      </c>
+      <c r="H5" s="8" t="n">
+        <v>0.4069</v>
+      </c>
+      <c r="I5" s="15" t="n">
+        <v>0.3918</v>
+      </c>
+      <c r="J5" s="14" t="n">
         <v>107460</v>
       </c>
-      <c r="G5" s="12" t="n">
+      <c r="K5" s="14" t="n">
         <v>29039</v>
       </c>
-      <c r="H5" s="8" t="n">
+      <c r="L5" s="9" t="n">
         <v>0.27</v>
       </c>
-      <c r="I5" s="12" t="n">
+      <c r="M5" s="14" t="n">
         <v>154375</v>
       </c>
-      <c r="J5" s="12" t="n">
+      <c r="N5" s="14" t="n">
         <v>2239216</v>
       </c>
-      <c r="K5" s="14" t="n">
+      <c r="O5" s="16" t="n">
         <v>2.46</v>
       </c>
-      <c r="L5" s="14" t="n">
+      <c r="P5" s="16" t="n">
         <v>1.23</v>
       </c>
-      <c r="M5" s="14" t="n">
+      <c r="Q5" s="16" t="n">
         <v>1.23</v>
       </c>
-      <c r="N5" s="10" t="n">
+      <c r="R5" s="11" t="n">
         <v>3.05</v>
       </c>
-      <c r="O5" s="12" t="n">
+      <c r="S5" s="14" t="n">
         <v>60000</v>
       </c>
-      <c r="P5" s="11" t="inlineStr">
+      <c r="T5" s="13" t="inlineStr">
         <is>
           <t>✅増分3.05・BC検証</t>
         </is>
       </c>
-      <c r="Q5" s="11" t="inlineStr">
-        <is>
-          <t>60k据置</t>
+      <c r="U5" s="17" t="inlineStr">
+        <is>
+          <t>①原価率18.9%は全商品で最良、広告費率40.7%が唯一の重し②増分MER3.05は合格ラインだがBC検証中のため本体増額は保留→BC判定後に60k→75kが第一候補③脱毛は通年需要。夏枯れの影響を受けない数少ない商品で、秋以降の主力候補</t>
         </is>
       </c>
     </row>
@@ -1351,103 +1452,129 @@
       <c r="E6" s="5" t="n">
         <v>335526</v>
       </c>
-      <c r="F6" s="5" t="n">
+      <c r="F6" s="6" t="n">
+        <v>0.4237</v>
+      </c>
+      <c r="G6" s="6" t="n">
+        <v>0.2612</v>
+      </c>
+      <c r="H6" s="6" t="n">
+        <v>0.3151</v>
+      </c>
+      <c r="I6" s="6" t="n">
+        <v>0.4058</v>
+      </c>
+      <c r="J6" s="5" t="n">
         <v>99600</v>
       </c>
-      <c r="G6" s="5" t="n">
+      <c r="K6" s="5" t="n">
         <v>33522</v>
       </c>
-      <c r="H6" s="6" t="n">
+      <c r="L6" s="6" t="n">
         <v>0.337</v>
       </c>
-      <c r="I6" s="5" t="n">
+      <c r="M6" s="5" t="n">
         <v>143494</v>
       </c>
-      <c r="J6" s="5" t="n">
+      <c r="N6" s="5" t="n">
         <v>939490</v>
       </c>
-      <c r="K6" s="9" t="n">
+      <c r="O6" s="10" t="n">
         <v>3.17</v>
       </c>
-      <c r="L6" s="9" t="n">
+      <c r="P6" s="10" t="n">
         <v>1.35</v>
       </c>
-      <c r="M6" s="9" t="n">
+      <c r="Q6" s="10" t="n">
         <v>1.82</v>
       </c>
-      <c r="N6" s="15" t="n">
+      <c r="R6" s="18" t="n">
         <v>2.46</v>
       </c>
-      <c r="O6" s="5" t="n">
+      <c r="S6" s="5" t="n">
         <v>41000</v>
       </c>
-      <c r="P6" s="4" t="inlineStr">
+      <c r="T6" s="4" t="inlineStr">
         <is>
           <t>👀7/28判定(増分2.46)</t>
         </is>
       </c>
-      <c r="Q6" s="4" t="inlineStr">
-        <is>
-          <t>41k据置</t>
+      <c r="U6" s="12" t="inlineStr">
+        <is>
+          <t>①増分MER2.46＝増額は利益率を下げる。41k据置が正解②7/28判定で2.91超なら50kへ③原価率26.1%・広告費率31.5%とも健全でボトルネックなし</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="11" t="inlineStr">
+      <c r="A7" s="13" t="inlineStr">
         <is>
           <t>卓上冷感クーラー</t>
         </is>
       </c>
-      <c r="B7" s="12" t="n">
+      <c r="B7" s="14" t="n">
         <v>765440</v>
       </c>
-      <c r="C7" s="12" t="n">
+      <c r="C7" s="14" t="n">
         <v>255488</v>
       </c>
-      <c r="D7" s="12" t="n">
+      <c r="D7" s="14" t="n">
         <v>180073</v>
       </c>
-      <c r="E7" s="12" t="n">
+      <c r="E7" s="14" t="n">
         <v>329879</v>
       </c>
-      <c r="F7" s="12" t="n">
+      <c r="F7" s="15" t="n">
+        <v>0.431</v>
+      </c>
+      <c r="G7" s="8" t="n">
+        <v>0.3338</v>
+      </c>
+      <c r="H7" s="15" t="n">
+        <v>0.2353</v>
+      </c>
+      <c r="I7" s="13" t="inlineStr">
+        <is>
+          <t>−</t>
+        </is>
+      </c>
+      <c r="J7" s="14" t="n">
         <v>125580</v>
       </c>
-      <c r="G7" s="12" t="n">
+      <c r="K7" s="14" t="n">
         <v>52218</v>
       </c>
-      <c r="H7" s="13" t="n">
+      <c r="L7" s="15" t="n">
         <v>0.416</v>
       </c>
-      <c r="I7" s="12" t="n">
+      <c r="M7" s="14" t="n">
         <v>199892</v>
       </c>
-      <c r="J7" s="12" t="n">
+      <c r="N7" s="14" t="n">
         <v>471963</v>
       </c>
-      <c r="K7" s="14" t="n">
+      <c r="O7" s="16" t="n">
         <v>4.25</v>
       </c>
-      <c r="L7" s="14" t="n">
+      <c r="P7" s="16" t="n">
         <v>1.5</v>
       </c>
-      <c r="M7" s="14" t="n">
+      <c r="Q7" s="16" t="n">
         <v>2.75</v>
       </c>
-      <c r="N7" s="10" t="n">
+      <c r="R7" s="11" t="n">
         <v>12.25</v>
       </c>
-      <c r="O7" s="12" t="n">
+      <c r="S7" s="14" t="n">
         <v>38000</v>
       </c>
-      <c r="P7" s="11" t="inlineStr">
+      <c r="T7" s="13" t="inlineStr">
         <is>
           <t>✅増分12.25(7/27判定)</t>
         </is>
       </c>
-      <c r="Q7" s="11" t="inlineStr">
-        <is>
-          <t>38k据置</t>
+      <c r="U7" s="17" t="inlineStr">
+        <is>
+          <t>①増分MER12.25は全商品最高だが消化率79%で38kを使い切れず。増額しても無意味②打ち手は「予算」ではなく「配信量」＝オーディエンス拡大かCR追加で配信面を広げる③原価率33.4%。売価5,980円で+500円値上げは11.2%減までOK④7/27に消化率85%超を確認</t>
         </is>
       </c>
     </row>
@@ -1469,103 +1596,129 @@
       <c r="E8" s="5" t="n">
         <v>253085</v>
       </c>
-      <c r="F8" s="5" t="n">
+      <c r="F8" s="6" t="n">
+        <v>0.3505</v>
+      </c>
+      <c r="G8" s="8" t="n">
+        <v>0.3614</v>
+      </c>
+      <c r="H8" s="6" t="n">
+        <v>0.2881</v>
+      </c>
+      <c r="I8" s="6" t="n">
+        <v>0.3194</v>
+      </c>
+      <c r="J8" s="5" t="n">
         <v>131340</v>
       </c>
-      <c r="G8" s="5" t="n">
+      <c r="K8" s="5" t="n">
         <v>51598</v>
       </c>
-      <c r="H8" s="6" t="n">
+      <c r="L8" s="6" t="n">
         <v>0.393</v>
       </c>
-      <c r="I8" s="5" t="n">
+      <c r="M8" s="5" t="n">
         <v>94073</v>
       </c>
-      <c r="J8" s="5" t="n">
+      <c r="N8" s="5" t="n">
         <v>754939</v>
       </c>
-      <c r="K8" s="9" t="n">
+      <c r="O8" s="10" t="n">
         <v>3.47</v>
       </c>
-      <c r="L8" s="9" t="n">
+      <c r="P8" s="10" t="n">
         <v>1.57</v>
       </c>
-      <c r="M8" s="9" t="n">
+      <c r="Q8" s="10" t="n">
         <v>1.9</v>
       </c>
-      <c r="N8" s="16" t="n">
+      <c r="R8" s="19" t="n">
         <v>-0.6</v>
       </c>
-      <c r="O8" s="5" t="n">
+      <c r="S8" s="5" t="n">
         <v>34000</v>
       </c>
-      <c r="P8" s="4" t="inlineStr">
+      <c r="T8" s="4" t="inlineStr">
         <is>
           <t>⚠️7/28判定(増分−0.60)</t>
         </is>
       </c>
-      <c r="Q8" s="4" t="inlineStr">
-        <is>
-          <t>34k据置</t>
+      <c r="U8" s="12" t="inlineStr">
+        <is>
+          <t>①増分MER−0.60。34k据置、7/28で改善なければ28kへ戻す②原価率36.1%が重い。売価3,980円と安く+500円値上げは16.4%減まで許容＝値上げ余地が最も大きい③3日利益率31.9%と7日35.0%より低下。CR疲弊の兆候→素材があれば投入</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="11" t="inlineStr">
+      <c r="A9" s="13" t="inlineStr">
         <is>
           <t>5WAY腰掛けファン</t>
         </is>
       </c>
-      <c r="B9" s="12" t="n">
+      <c r="B9" s="14" t="n">
         <v>333660</v>
       </c>
-      <c r="C9" s="12" t="n">
+      <c r="C9" s="14" t="n">
         <v>123816</v>
       </c>
-      <c r="D9" s="12" t="n">
+      <c r="D9" s="14" t="n">
         <v>64413</v>
       </c>
-      <c r="E9" s="12" t="n">
+      <c r="E9" s="14" t="n">
         <v>145431</v>
       </c>
-      <c r="F9" s="12" t="n">
+      <c r="F9" s="15" t="n">
+        <v>0.4359</v>
+      </c>
+      <c r="G9" s="8" t="n">
+        <v>0.3711</v>
+      </c>
+      <c r="H9" s="15" t="n">
+        <v>0.193</v>
+      </c>
+      <c r="I9" s="13" t="inlineStr">
+        <is>
+          <t>−</t>
+        </is>
+      </c>
+      <c r="J9" s="14" t="n">
         <v>39840</v>
       </c>
-      <c r="G9" s="12" t="n">
+      <c r="K9" s="14" t="n">
         <v>13211</v>
       </c>
-      <c r="H9" s="13" t="n">
+      <c r="L9" s="15" t="n">
         <v>0.332</v>
       </c>
-      <c r="I9" s="12" t="n">
+      <c r="M9" s="14" t="n">
         <v>59969</v>
       </c>
-      <c r="J9" s="12" t="n">
+      <c r="N9" s="14" t="n">
         <v>145431</v>
       </c>
-      <c r="K9" s="14" t="n">
+      <c r="O9" s="16" t="n">
         <v>5.18</v>
       </c>
-      <c r="L9" s="14" t="n">
+      <c r="P9" s="16" t="n">
         <v>1.59</v>
       </c>
-      <c r="M9" s="14" t="n">
+      <c r="Q9" s="16" t="n">
         <v>3.59</v>
       </c>
-      <c r="N9" s="15" t="n">
+      <c r="R9" s="18" t="n">
         <v>1.85</v>
       </c>
-      <c r="O9" s="12" t="n">
+      <c r="S9" s="14" t="n">
         <v>13000</v>
       </c>
-      <c r="P9" s="11" t="inlineStr">
+      <c r="T9" s="13" t="inlineStr">
         <is>
           <t>👀7/28判定(増分1.85・学習中)</t>
         </is>
       </c>
-      <c r="Q9" s="11" t="inlineStr">
-        <is>
-          <t>13k据置</t>
+      <c r="U9" s="17" t="inlineStr">
+        <is>
+          <t>①増分MER1.85・学習中。13k据置②広告費率19.3%は最良＝伸ばす余地が最も大きい。学習完了後の増額最有力③原価率37.1%が唯一の弱点。売価4,980円で+500円値上げは13.8%減までOK</t>
         </is>
       </c>
     </row>
@@ -1587,99 +1740,127 @@
       <c r="E10" s="5" t="n">
         <v>95178</v>
       </c>
-      <c r="F10" s="5" t="n">
+      <c r="F10" s="9" t="n">
+        <v>0.2959</v>
+      </c>
+      <c r="G10" s="6" t="n">
+        <v>0.2249</v>
+      </c>
+      <c r="H10" s="8" t="n">
+        <v>0.4793</v>
+      </c>
+      <c r="I10" s="4" t="inlineStr">
+        <is>
+          <t>−</t>
+        </is>
+      </c>
+      <c r="J10" s="5" t="n">
         <v>43780</v>
       </c>
-      <c r="G10" s="5" t="n">
+      <c r="K10" s="5" t="n">
         <v>13552</v>
       </c>
-      <c r="H10" s="6" t="n">
+      <c r="L10" s="6" t="n">
         <v>0.31</v>
       </c>
-      <c r="I10" s="5" t="n">
+      <c r="M10" s="5" t="n">
         <v>28693</v>
       </c>
-      <c r="J10" s="5" t="n">
+      <c r="N10" s="5" t="n">
         <v>576804</v>
       </c>
-      <c r="K10" s="9" t="n">
+      <c r="O10" s="10" t="n">
         <v>2.09</v>
       </c>
-      <c r="L10" s="9" t="n">
+      <c r="P10" s="10" t="n">
         <v>1.29</v>
       </c>
-      <c r="M10" s="9" t="n">
+      <c r="Q10" s="10" t="n">
         <v>0.8</v>
       </c>
-      <c r="N10" s="4" t="inlineStr"/>
-      <c r="O10" s="5" t="n">
+      <c r="R10" s="4" t="inlineStr"/>
+      <c r="S10" s="5" t="n">
         <v>22000</v>
       </c>
-      <c r="P10" s="4" t="inlineStr">
+      <c r="T10" s="4" t="inlineStr">
         <is>
           <t>⚠️先行指標継続(持越)</t>
         </is>
       </c>
-      <c r="Q10" s="4" t="inlineStr">
-        <is>
-          <t>22k維持</t>
+      <c r="U10" s="12" t="inlineStr">
+        <is>
+          <t>①広告費率47.9%が主因。原価率22.5%は健全＝広告の問題②余裕+0.80で増額ラインに届かず、余裕&gt;0なので減額もしない→CR/LPで手当て③増分MER判定保留。次に予算を動かすときは±25%以上（22k→27k or 17k）動かして測定可能にする④7/29を判定日に新設</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="11" t="inlineStr">
+      <c r="A11" s="13" t="inlineStr">
         <is>
           <t>3WAYサーキュレーター扇風機</t>
         </is>
       </c>
-      <c r="B11" s="12" t="n">
+      <c r="B11" s="14" t="n">
         <v>316940</v>
       </c>
-      <c r="C11" s="12" t="n">
+      <c r="C11" s="14" t="n">
         <v>131705</v>
       </c>
-      <c r="D11" s="12" t="n">
+      <c r="D11" s="14" t="n">
         <v>96961</v>
       </c>
-      <c r="E11" s="12" t="n">
+      <c r="E11" s="14" t="n">
         <v>88274</v>
       </c>
-      <c r="F11" s="12" t="n">
+      <c r="F11" s="9" t="n">
+        <v>0.2785</v>
+      </c>
+      <c r="G11" s="8" t="n">
+        <v>0.4156</v>
+      </c>
+      <c r="H11" s="15" t="n">
+        <v>0.3059</v>
+      </c>
+      <c r="I11" s="13" t="inlineStr">
+        <is>
+          <t>−</t>
+        </is>
+      </c>
+      <c r="J11" s="14" t="n">
         <v>11960</v>
       </c>
-      <c r="G11" s="17" t="n">
+      <c r="K11" s="20" t="n">
         <v>-8824</v>
       </c>
-      <c r="H11" s="8" t="n">
+      <c r="L11" s="21" t="n">
         <v>-0.738</v>
       </c>
-      <c r="I11" s="12" t="n">
+      <c r="M11" s="14" t="n">
         <v>35832</v>
       </c>
-      <c r="J11" s="12" t="n">
+      <c r="N11" s="14" t="n">
         <v>239361</v>
       </c>
-      <c r="K11" s="14" t="n">
+      <c r="O11" s="16" t="n">
         <v>3.27</v>
       </c>
-      <c r="L11" s="14" t="n">
+      <c r="P11" s="16" t="n">
         <v>1.71</v>
       </c>
-      <c r="M11" s="14" t="n">
+      <c r="Q11" s="16" t="n">
         <v>1.56</v>
       </c>
-      <c r="N11" s="11" t="inlineStr"/>
-      <c r="O11" s="12" t="n">
+      <c r="R11" s="13" t="inlineStr"/>
+      <c r="S11" s="14" t="n">
         <v>16000</v>
       </c>
-      <c r="P11" s="11" t="inlineStr">
+      <c r="T11" s="13" t="inlineStr">
         <is>
           <t>✅増額判定: 据置(3日MER3.09)</t>
         </is>
       </c>
-      <c r="Q11" s="11" t="inlineStr">
-        <is>
-          <t>16k維持</t>
+      <c r="U11" s="17" t="inlineStr">
+        <is>
+          <t>①原価率41.6%が主因。広告ではなく原価か価格の問題②売価5,980円で+1,000円値上げは22.2%減まで許容＝値上げの最有力候補③CJに原価交渉（2,485円→2,200円で原価率36.8%・利益率+4.8pt）④日販7.6個で利益率がブレるため7日累計で判断</t>
         </is>
       </c>
     </row>
@@ -1701,101 +1882,129 @@
       <c r="E12" s="5" t="n">
         <v>71635</v>
       </c>
-      <c r="F12" s="5" t="n">
+      <c r="F12" s="6" t="n">
+        <v>0.3002</v>
+      </c>
+      <c r="G12" s="6" t="n">
+        <v>0.1971</v>
+      </c>
+      <c r="H12" s="8" t="n">
+        <v>0.5027</v>
+      </c>
+      <c r="I12" s="4" t="inlineStr">
+        <is>
+          <t>−</t>
+        </is>
+      </c>
+      <c r="J12" s="5" t="n">
         <v>31840</v>
       </c>
-      <c r="G12" s="5" t="n">
+      <c r="K12" s="5" t="n">
         <v>8342</v>
       </c>
-      <c r="H12" s="8" t="n">
+      <c r="L12" s="9" t="n">
         <v>0.262</v>
       </c>
-      <c r="I12" s="5" t="n">
+      <c r="M12" s="5" t="n">
         <v>25739</v>
       </c>
-      <c r="J12" s="5" t="n">
+      <c r="N12" s="5" t="n">
         <v>389240</v>
       </c>
-      <c r="K12" s="9" t="n">
+      <c r="O12" s="10" t="n">
         <v>1.99</v>
       </c>
-      <c r="L12" s="9" t="n">
+      <c r="P12" s="10" t="n">
         <v>1.25</v>
       </c>
-      <c r="M12" s="9" t="n">
+      <c r="Q12" s="10" t="n">
         <v>0.74</v>
       </c>
-      <c r="N12" s="4" t="inlineStr"/>
-      <c r="O12" s="5" t="n">
+      <c r="R12" s="4" t="inlineStr"/>
+      <c r="S12" s="5" t="n">
         <v>17000</v>
       </c>
-      <c r="P12" s="4" t="inlineStr">
+      <c r="T12" s="4" t="inlineStr">
         <is>
           <t>✅維持</t>
         </is>
       </c>
-      <c r="Q12" s="4" t="inlineStr">
-        <is>
-          <t>17k維持</t>
+      <c r="U12" s="12" t="inlineStr">
+        <is>
+          <t>①広告費率50.3%が主因。原価率19.7%は極めて良い②売価3,980円と低くAOVが小さいのが構造要因→パーカー/UVハットとのセット販売でAOVを上げるのが本命③余裕+0.74で増減いずれもしない。CR/クロスセルで手当て④7/29を判定日に新設</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="11" t="inlineStr">
+      <c r="A13" s="13" t="inlineStr">
         <is>
           <t>ムダ毛シェーバー</t>
         </is>
       </c>
-      <c r="B13" s="12" t="n">
+      <c r="B13" s="14" t="n">
         <v>215280</v>
       </c>
-      <c r="C13" s="12" t="n">
+      <c r="C13" s="14" t="n">
         <v>100728</v>
       </c>
-      <c r="D13" s="12" t="n">
+      <c r="D13" s="14" t="n">
         <v>92441</v>
       </c>
-      <c r="E13" s="12" t="n">
+      <c r="E13" s="14" t="n">
         <v>22111</v>
       </c>
-      <c r="F13" s="12" t="n">
+      <c r="F13" s="9" t="n">
+        <v>0.1027</v>
+      </c>
+      <c r="G13" s="8" t="n">
+        <v>0.4679</v>
+      </c>
+      <c r="H13" s="8" t="n">
+        <v>0.4294</v>
+      </c>
+      <c r="I13" s="13" t="inlineStr">
+        <is>
+          <t>−</t>
+        </is>
+      </c>
+      <c r="J13" s="14" t="n">
         <v>29900</v>
       </c>
-      <c r="G13" s="12" t="n">
+      <c r="K13" s="14" t="n">
         <v>4611</v>
       </c>
-      <c r="H13" s="8" t="n">
+      <c r="L13" s="9" t="n">
         <v>0.154</v>
       </c>
-      <c r="I13" s="12" t="n">
+      <c r="M13" s="14" t="n">
         <v>17139</v>
       </c>
-      <c r="J13" s="12" t="n">
+      <c r="N13" s="14" t="n">
         <v>48109</v>
       </c>
-      <c r="K13" s="14" t="n">
+      <c r="O13" s="16" t="n">
         <v>2.33</v>
       </c>
-      <c r="L13" s="14" t="n">
+      <c r="P13" s="16" t="n">
         <v>1.88</v>
       </c>
-      <c r="M13" s="14" t="n">
+      <c r="Q13" s="16" t="n">
         <v>0.45</v>
       </c>
-      <c r="N13" s="16" t="n">
+      <c r="R13" s="19" t="n">
         <v>-1.24</v>
       </c>
-      <c r="O13" s="12" t="n">
+      <c r="S13" s="14" t="n">
         <v>13000</v>
       </c>
-      <c r="P13" s="11" t="inlineStr">
+      <c r="T13" s="13" t="inlineStr">
         <is>
           <t>🔧減額が正解(増分−1.24)8/1</t>
         </is>
       </c>
-      <c r="Q13" s="11" t="inlineStr">
-        <is>
-          <t>13k据置</t>
+      <c r="U13" s="17" t="inlineStr">
+        <is>
+          <t>①原価率46.8%が最大の問題。広告をいじっても直らない②売価5,980円で+1,000円値上げは23.9%減まで許容＝値上げの最優先候補③CJに原価交渉（2,798円は7/25改定でも据置＝交渉余地あり）④増分MER−1.24＝減額しても売上が落ちない。7/27判定で13k→10kも選択肢</t>
         </is>
       </c>
     </row>
@@ -1817,99 +2026,127 @@
       <c r="E14" s="5" t="n">
         <v>46436</v>
       </c>
-      <c r="F14" s="5" t="n">
+      <c r="F14" s="9" t="n">
+        <v>0.2605</v>
+      </c>
+      <c r="G14" s="6" t="n">
+        <v>0.2281</v>
+      </c>
+      <c r="H14" s="8" t="n">
+        <v>0.5114</v>
+      </c>
+      <c r="I14" s="4" t="inlineStr">
+        <is>
+          <t>−</t>
+        </is>
+      </c>
+      <c r="J14" s="5" t="n">
         <v>24900</v>
       </c>
-      <c r="G14" s="5" t="n">
+      <c r="K14" s="5" t="n">
         <v>5784</v>
       </c>
-      <c r="H14" s="8" t="n">
+      <c r="L14" s="9" t="n">
         <v>0.232</v>
       </c>
-      <c r="I14" s="5" t="n">
+      <c r="M14" s="5" t="n">
         <v>27274</v>
       </c>
-      <c r="J14" s="5" t="n">
+      <c r="N14" s="5" t="n">
         <v>320995</v>
       </c>
-      <c r="K14" s="9" t="n">
+      <c r="O14" s="10" t="n">
         <v>1.96</v>
       </c>
-      <c r="L14" s="9" t="n">
+      <c r="P14" s="10" t="n">
         <v>1.3</v>
       </c>
-      <c r="M14" s="9" t="n">
+      <c r="Q14" s="10" t="n">
         <v>0.66</v>
       </c>
-      <c r="N14" s="4" t="inlineStr"/>
-      <c r="O14" s="5" t="n">
+      <c r="R14" s="4" t="inlineStr"/>
+      <c r="S14" s="5" t="n">
         <v>13000</v>
       </c>
-      <c r="P14" s="4" t="inlineStr">
+      <c r="T14" s="4" t="inlineStr">
         <is>
           <t>👀弱含み</t>
         </is>
       </c>
-      <c r="Q14" s="4" t="inlineStr">
-        <is>
-          <t>13k維持</t>
+      <c r="U14" s="12" t="inlineStr">
+        <is>
+          <t>①広告費率51.1%が主因。原価率22.8%は良好②売価4,980円・日販5個。サイズ展開18種で在庫リスクは無いがCVRが低い→LP/サイズ選択UIの改善が本命③余裕+0.66。増減せずCR差し替え④秋以降も需要継続する数少ない非季節商品</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="11" t="inlineStr">
+      <c r="A15" s="13" t="inlineStr">
         <is>
           <t>瞬間冷感ポンチョ</t>
         </is>
       </c>
-      <c r="B15" s="12" t="n">
+      <c r="B15" s="14" t="n">
         <v>159200</v>
       </c>
-      <c r="C15" s="12" t="n">
+      <c r="C15" s="14" t="n">
         <v>39480</v>
       </c>
-      <c r="D15" s="12" t="n">
+      <c r="D15" s="14" t="n">
         <v>91828</v>
       </c>
-      <c r="E15" s="12" t="n">
+      <c r="E15" s="14" t="n">
         <v>27892</v>
       </c>
-      <c r="F15" s="12" t="n">
+      <c r="F15" s="9" t="n">
+        <v>0.1752</v>
+      </c>
+      <c r="G15" s="15" t="n">
+        <v>0.248</v>
+      </c>
+      <c r="H15" s="8" t="n">
+        <v>0.5768</v>
+      </c>
+      <c r="I15" s="13" t="inlineStr">
+        <is>
+          <t>−</t>
+        </is>
+      </c>
+      <c r="J15" s="14" t="n">
         <v>47760</v>
       </c>
-      <c r="G15" s="12" t="n">
+      <c r="K15" s="14" t="n">
         <v>24112</v>
       </c>
-      <c r="H15" s="13" t="n">
+      <c r="L15" s="15" t="n">
         <v>0.505</v>
       </c>
-      <c r="I15" s="12" t="n">
+      <c r="M15" s="14" t="n">
         <v>51827</v>
       </c>
-      <c r="J15" s="12" t="n">
+      <c r="N15" s="14" t="n">
         <v>125094</v>
       </c>
-      <c r="K15" s="14" t="n">
+      <c r="O15" s="16" t="n">
         <v>1.73</v>
       </c>
-      <c r="L15" s="14" t="n">
+      <c r="P15" s="16" t="n">
         <v>1.33</v>
       </c>
-      <c r="M15" s="14" t="n">
+      <c r="Q15" s="16" t="n">
         <v>0.4</v>
       </c>
-      <c r="N15" s="11" t="inlineStr"/>
-      <c r="O15" s="12" t="n">
+      <c r="R15" s="13" t="inlineStr"/>
+      <c r="S15" s="14" t="n">
         <v>13000</v>
       </c>
-      <c r="P15" s="11" t="inlineStr">
+      <c r="T15" s="13" t="inlineStr">
         <is>
           <t>✅維持</t>
         </is>
       </c>
-      <c r="Q15" s="11" t="inlineStr">
-        <is>
-          <t>13k維持</t>
+      <c r="U15" s="17" t="inlineStr">
+        <is>
+          <t>①広告費率57.7%が主因で利益率17.5%と低い②増分MER判定保留。13k→10kに下げて増分を測るのが有効（−3,000円で測定可能に）③夏物の中で最も季節性が強い。8月中旬から真っ先に縮小する対象④原価率24.8%は良好なので、需要期に効率が戻れば伸ばせる</t>
         </is>
       </c>
     </row>
@@ -1931,99 +2168,127 @@
       <c r="E16" s="5" t="n">
         <v>16972</v>
       </c>
-      <c r="F16" s="5" t="n">
+      <c r="F16" s="9" t="n">
+        <v>0.1175</v>
+      </c>
+      <c r="G16" s="8" t="n">
+        <v>0.3379</v>
+      </c>
+      <c r="H16" s="8" t="n">
+        <v>0.5446</v>
+      </c>
+      <c r="I16" s="4" t="inlineStr">
+        <is>
+          <t>−</t>
+        </is>
+      </c>
+      <c r="J16" s="5" t="n">
         <v>4980</v>
       </c>
-      <c r="G16" s="18" t="n">
+      <c r="K16" s="22" t="n">
         <v>-7092</v>
       </c>
-      <c r="H16" s="8" t="n">
+      <c r="L16" s="21" t="n">
         <v>-1.424</v>
       </c>
-      <c r="I16" s="18" t="n">
+      <c r="M16" s="22" t="n">
         <v>-652</v>
       </c>
-      <c r="J16" s="5" t="n">
+      <c r="N16" s="5" t="n">
         <v>220759</v>
       </c>
-      <c r="K16" s="9" t="n">
+      <c r="O16" s="10" t="n">
         <v>1.84</v>
       </c>
-      <c r="L16" s="9" t="n">
+      <c r="P16" s="10" t="n">
         <v>1.51</v>
       </c>
-      <c r="M16" s="9" t="n">
+      <c r="Q16" s="10" t="n">
         <v>0.33</v>
       </c>
-      <c r="N16" s="4" t="inlineStr"/>
-      <c r="O16" s="5" t="n">
+      <c r="R16" s="4" t="inlineStr"/>
+      <c r="S16" s="5" t="n">
         <v>11000</v>
       </c>
-      <c r="P16" s="4" t="inlineStr">
+      <c r="T16" s="4" t="inlineStr">
         <is>
           <t>👀前日弱</t>
         </is>
       </c>
-      <c r="Q16" s="4" t="inlineStr">
-        <is>
-          <t>11k維持</t>
+      <c r="U16" s="12" t="inlineStr">
+        <is>
+          <t>①広告費率54.5%・原価率33.8%の両方が重い②日販4個で利益率のブレが±64pt＝利益率では判断不能。7日累計利益16,972円（黒字）で見る③8/1判定。余裕+0.33と薄く、7日が赤字転落したら即減額④売価4,980円で+500円値上げは13.4%減まで許容</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="11" t="inlineStr">
+      <c r="A17" s="13" t="inlineStr">
         <is>
           <t>UV歯ブラシ除菌器</t>
         </is>
       </c>
-      <c r="B17" s="12" t="n">
+      <c r="B17" s="14" t="n">
         <v>125720</v>
       </c>
-      <c r="C17" s="12" t="n">
+      <c r="C17" s="14" t="n">
         <v>45360</v>
       </c>
-      <c r="D17" s="12" t="n">
+      <c r="D17" s="14" t="n">
         <v>85489</v>
       </c>
-      <c r="E17" s="17" t="n">
+      <c r="E17" s="20" t="n">
         <v>-5129</v>
       </c>
-      <c r="F17" s="12" t="n">
+      <c r="F17" s="21" t="n">
+        <v>-0.0408</v>
+      </c>
+      <c r="G17" s="8" t="n">
+        <v>0.3608</v>
+      </c>
+      <c r="H17" s="8" t="n">
+        <v>0.68</v>
+      </c>
+      <c r="I17" s="13" t="inlineStr">
+        <is>
+          <t>−</t>
+        </is>
+      </c>
+      <c r="J17" s="14" t="n">
         <v>35920</v>
       </c>
-      <c r="G17" s="12" t="n">
+      <c r="K17" s="14" t="n">
         <v>13193</v>
       </c>
-      <c r="H17" s="13" t="n">
+      <c r="L17" s="15" t="n">
         <v>0.367</v>
       </c>
-      <c r="I17" s="12" t="n">
+      <c r="M17" s="14" t="n">
         <v>1425</v>
       </c>
-      <c r="J17" s="12" t="n">
+      <c r="N17" s="14" t="n">
         <v>267661</v>
       </c>
-      <c r="K17" s="14" t="n">
+      <c r="O17" s="16" t="n">
         <v>1.47</v>
       </c>
-      <c r="L17" s="14" t="n">
+      <c r="P17" s="16" t="n">
         <v>1.56</v>
       </c>
-      <c r="M17" s="14" t="n">
+      <c r="Q17" s="16" t="n">
         <v>-0.09</v>
       </c>
-      <c r="N17" s="11" t="inlineStr"/>
-      <c r="O17" s="12" t="n">
+      <c r="R17" s="13" t="inlineStr"/>
+      <c r="S17" s="14" t="n">
         <v>10000</v>
       </c>
-      <c r="P17" s="11" t="inlineStr">
+      <c r="T17" s="13" t="inlineStr">
         <is>
           <t>🔧複製リセット中(7/30)</t>
         </is>
       </c>
-      <c r="Q17" s="11" t="inlineStr">
-        <is>
-          <t>10k据置</t>
+      <c r="U17" s="17" t="inlineStr">
+        <is>
+          <t>①広告費率68.0%＝完全に広告過多。原価率36.1%も重い②3日利益+1,425円で黒字転換の兆し＝複製リセットが効き始めた可能性③7/30判定。改善なければ10k→6kへ半減④売価8,980円は最高単価。+500円値上げは8.0%減までしか許容できず値上げ余地は小さい</t>
         </is>
       </c>
     </row>
@@ -2042,106 +2307,134 @@
       <c r="D18" s="5" t="n">
         <v>94262</v>
       </c>
-      <c r="E18" s="18" t="n">
+      <c r="E18" s="22" t="n">
         <v>-29294</v>
       </c>
-      <c r="F18" s="5" t="n">
+      <c r="F18" s="21" t="n">
+        <v>-0.2909</v>
+      </c>
+      <c r="G18" s="8" t="n">
+        <v>0.3548</v>
+      </c>
+      <c r="H18" s="8" t="n">
+        <v>0.9361</v>
+      </c>
+      <c r="I18" s="4" t="inlineStr">
+        <is>
+          <t>−</t>
+        </is>
+      </c>
+      <c r="J18" s="5" t="n">
         <v>12960</v>
       </c>
-      <c r="G18" s="18" t="n">
+      <c r="K18" s="22" t="n">
         <v>-2390</v>
       </c>
-      <c r="H18" s="8" t="n">
+      <c r="L18" s="21" t="n">
         <v>-0.184</v>
       </c>
-      <c r="I18" s="18" t="n">
+      <c r="M18" s="22" t="n">
         <v>-14004</v>
       </c>
-      <c r="J18" s="5" t="n">
+      <c r="N18" s="5" t="n">
         <v>123009</v>
       </c>
-      <c r="K18" s="9" t="n">
+      <c r="O18" s="10" t="n">
         <v>1.07</v>
       </c>
-      <c r="L18" s="9" t="n">
+      <c r="P18" s="10" t="n">
         <v>1.55</v>
       </c>
-      <c r="M18" s="9" t="n">
+      <c r="Q18" s="10" t="n">
         <v>-0.48</v>
       </c>
-      <c r="N18" s="15" t="n">
+      <c r="R18" s="18" t="n">
         <v>1.82</v>
       </c>
-      <c r="O18" s="5" t="n">
+      <c r="S18" s="5" t="n">
         <v>12000</v>
       </c>
-      <c r="P18" s="4" t="inlineStr">
+      <c r="T18" s="4" t="inlineStr">
         <is>
           <t>🚨全開放テスト(8/6)</t>
         </is>
       </c>
-      <c r="Q18" s="4" t="inlineStr">
-        <is>
-          <t>6k+6k据置</t>
+      <c r="U18" s="12" t="inlineStr">
+        <is>
+          <t>①広告費率93.6%＝売上のほぼ全額が広告費。構造的に成立していない②本日、類似5%を停止し全開放6kのみに（12k→6k）③8/1にCPA&gt;6,000なら早期停止、8/6最終判定④週50CVに必要な予算44,887円/日は出せない＝学習を抜けられない構造問題</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="11" t="inlineStr">
+      <c r="A19" s="13" t="inlineStr">
         <is>
           <t>バランスケアスリッパ</t>
         </is>
       </c>
-      <c r="B19" s="12" t="n">
+      <c r="B19" s="14" t="n">
         <v>84660</v>
       </c>
-      <c r="C19" s="12" t="n">
+      <c r="C19" s="14" t="n">
         <v>22168</v>
       </c>
-      <c r="D19" s="12" t="n">
+      <c r="D19" s="14" t="n">
         <v>57798</v>
       </c>
-      <c r="E19" s="12" t="n">
+      <c r="E19" s="14" t="n">
         <v>4694</v>
       </c>
-      <c r="F19" s="12" t="n">
+      <c r="F19" s="9" t="n">
+        <v>0.0554</v>
+      </c>
+      <c r="G19" s="15" t="n">
+        <v>0.2618</v>
+      </c>
+      <c r="H19" s="8" t="n">
+        <v>0.6827</v>
+      </c>
+      <c r="I19" s="13" t="inlineStr">
+        <is>
+          <t>−</t>
+        </is>
+      </c>
+      <c r="J19" s="14" t="n">
         <v>4980</v>
       </c>
-      <c r="G19" s="17" t="n">
+      <c r="K19" s="20" t="n">
         <v>-1553</v>
       </c>
-      <c r="H19" s="8" t="n">
+      <c r="L19" s="21" t="n">
         <v>-0.312</v>
       </c>
-      <c r="I19" s="12" t="n">
+      <c r="M19" s="14" t="n">
         <v>8072</v>
       </c>
-      <c r="J19" s="12" t="n">
+      <c r="N19" s="14" t="n">
         <v>94581</v>
       </c>
-      <c r="K19" s="14" t="n">
+      <c r="O19" s="16" t="n">
         <v>1.46</v>
       </c>
-      <c r="L19" s="14" t="n">
+      <c r="P19" s="16" t="n">
         <v>1.35</v>
       </c>
-      <c r="M19" s="14" t="n">
+      <c r="Q19" s="16" t="n">
         <v>0.11</v>
       </c>
-      <c r="N19" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="O19" s="12" t="n">
+      <c r="R19" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="S19" s="14" t="n">
         <v>5000</v>
       </c>
-      <c r="P19" s="11" t="inlineStr">
+      <c r="T19" s="13" t="inlineStr">
         <is>
           <t>🔧減額が正解(増分0.00)7/29</t>
         </is>
       </c>
-      <c r="Q19" s="11" t="inlineStr">
-        <is>
-          <t>5k据置</t>
+      <c r="U19" s="17" t="inlineStr">
+        <is>
+          <t>①広告費率68.3%。原価率26.2%は良好で広告の問題②増分MER0.00＝減らしても売上が落ちない。7/29判定で5k→3kかCR差し替え③日販2.4個。利益率でなく7日累計（+4,694円）で判断④非季節商品なので秋以降も継続可能</t>
         </is>
       </c>
     </row>
@@ -2160,94 +2453,122 @@
       <c r="D20" s="5" t="n">
         <v>56119</v>
       </c>
-      <c r="E20" s="18" t="n">
+      <c r="E20" s="22" t="n">
         <v>-2951</v>
       </c>
-      <c r="F20" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="G20" s="18" t="n">
+      <c r="F20" s="21" t="n">
+        <v>-0.0366</v>
+      </c>
+      <c r="G20" s="8" t="n">
+        <v>0.3413</v>
+      </c>
+      <c r="H20" s="8" t="n">
+        <v>0.6952</v>
+      </c>
+      <c r="I20" s="4" t="inlineStr">
+        <is>
+          <t>−</t>
+        </is>
+      </c>
+      <c r="J20" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="K20" s="22" t="n">
         <v>-6289</v>
       </c>
-      <c r="H20" s="4" t="inlineStr"/>
-      <c r="I20" s="18" t="n">
+      <c r="L20" s="4" t="inlineStr"/>
+      <c r="M20" s="22" t="n">
         <v>-6539</v>
       </c>
-      <c r="J20" s="5" t="n">
+      <c r="N20" s="5" t="n">
         <v>108918</v>
       </c>
-      <c r="K20" s="9" t="n">
+      <c r="O20" s="10" t="n">
         <v>1.44</v>
       </c>
-      <c r="L20" s="9" t="n">
+      <c r="P20" s="10" t="n">
         <v>1.52</v>
       </c>
-      <c r="M20" s="9" t="n">
+      <c r="Q20" s="10" t="n">
         <v>-0.08</v>
       </c>
-      <c r="N20" s="10" t="n">
+      <c r="R20" s="11" t="n">
         <v>2.91</v>
       </c>
-      <c r="O20" s="5" t="n">
+      <c r="S20" s="5" t="n">
         <v>6500</v>
       </c>
-      <c r="P20" s="4" t="inlineStr">
+      <c r="T20" s="4" t="inlineStr">
         <is>
           <t>🔧段階②判定は7/26</t>
         </is>
       </c>
-      <c r="Q20" s="4" t="inlineStr">
-        <is>
-          <t>6.5k据置</t>
+      <c r="U20" s="12" t="inlineStr">
+        <is>
+          <t>①広告費率69.5%で赤字。原価率34.1%も重い②明日7/26が段階②判定。7日余裕≥+0.3を満たさなければ停止③売価5,980円で+1,000円値上げは20.0%減まで許容だが、赤字商品の値上げは需要をさらに削る＝先に広告を絞るべき④夏物のため9月以降の継続価値は低い</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="11" t="inlineStr">
+      <c r="A21" s="13" t="inlineStr">
         <is>
           <t>瞬間冷却ハンディファン</t>
         </is>
       </c>
-      <c r="B21" s="12" t="n">
+      <c r="B21" s="14" t="n">
         <v>47840</v>
       </c>
-      <c r="C21" s="12" t="n">
+      <c r="C21" s="14" t="n">
         <v>16424</v>
       </c>
-      <c r="D21" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="E21" s="12" t="n">
+      <c r="D21" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="E21" s="14" t="n">
         <v>31416</v>
       </c>
-      <c r="F21" s="12" t="n">
+      <c r="F21" s="15" t="n">
+        <v>0.6567</v>
+      </c>
+      <c r="G21" s="8" t="n">
+        <v>0.3433</v>
+      </c>
+      <c r="H21" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="I21" s="13" t="inlineStr">
+        <is>
+          <t>−</t>
+        </is>
+      </c>
+      <c r="J21" s="14" t="n">
         <v>5980</v>
       </c>
-      <c r="G21" s="12" t="n">
+      <c r="K21" s="14" t="n">
         <v>3927</v>
       </c>
-      <c r="H21" s="13" t="n">
+      <c r="L21" s="15" t="n">
         <v>0.657</v>
       </c>
-      <c r="I21" s="12" t="n">
+      <c r="M21" s="14" t="n">
         <v>19635</v>
       </c>
-      <c r="J21" s="12" t="n">
+      <c r="N21" s="14" t="n">
         <v>70686</v>
       </c>
-      <c r="K21" s="11" t="inlineStr"/>
-      <c r="L21" s="11" t="inlineStr"/>
-      <c r="M21" s="11" t="inlineStr"/>
-      <c r="N21" s="11" t="inlineStr"/>
-      <c r="O21" s="11" t="inlineStr"/>
-      <c r="P21" s="11" t="inlineStr">
+      <c r="O21" s="13" t="inlineStr"/>
+      <c r="P21" s="13" t="inlineStr"/>
+      <c r="Q21" s="13" t="inlineStr"/>
+      <c r="R21" s="13" t="inlineStr"/>
+      <c r="S21" s="13" t="inlineStr"/>
+      <c r="T21" s="13" t="inlineStr">
         <is>
           <t>📦広告なし</t>
         </is>
       </c>
-      <c r="Q21" s="11" t="inlineStr">
-        <is>
-          <t>−</t>
+      <c r="U21" s="17" t="inlineStr">
+        <is>
+          <t>①広告ゼロで7日3.1万円の利益＝完全な粗利。4WAYからの流入と推定②広告を出す判断はしない（4WAYと共食いになる）③在庫消化用として現状維持</t>
         </is>
       </c>
     </row>
@@ -2269,81 +2590,109 @@
       <c r="E22" s="5" t="n">
         <v>42880</v>
       </c>
-      <c r="F22" s="5" t="n">
+      <c r="F22" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="G22" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H22" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I22" s="4" t="inlineStr">
+        <is>
+          <t>−</t>
+        </is>
+      </c>
+      <c r="J22" s="5" t="n">
         <v>6432</v>
       </c>
-      <c r="G22" s="5" t="n">
+      <c r="K22" s="5" t="n">
         <v>6432</v>
       </c>
-      <c r="H22" s="6" t="n">
+      <c r="L22" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="I22" s="5" t="n">
+      <c r="M22" s="5" t="n">
         <v>18224</v>
       </c>
-      <c r="J22" s="5" t="n">
+      <c r="N22" s="5" t="n">
         <v>110952</v>
       </c>
-      <c r="K22" s="4" t="inlineStr"/>
-      <c r="L22" s="4" t="inlineStr"/>
-      <c r="M22" s="4" t="inlineStr"/>
-      <c r="N22" s="4" t="inlineStr"/>
       <c r="O22" s="4" t="inlineStr"/>
-      <c r="P22" s="4" t="inlineStr">
+      <c r="P22" s="4" t="inlineStr"/>
+      <c r="Q22" s="4" t="inlineStr"/>
+      <c r="R22" s="4" t="inlineStr"/>
+      <c r="S22" s="4" t="inlineStr"/>
+      <c r="T22" s="4" t="inlineStr">
         <is>
           <t>📦広告なし</t>
         </is>
       </c>
-      <c r="Q22" s="4" t="inlineStr">
+      <c r="U22" s="12" t="inlineStr">
+        <is>
+          <t>①アタッチ率3.49%（80件/2,289注文）。原価0＝売上全額が利益②〜3,980円の注文230件でアタッチ0%＝590円が注文額の14.8%で高すぎる③商品説明に具体的な日数を入れる（現在「早くお届け」のみ）④低単価帯だけ390円にする段階価格をテスト</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="13" t="inlineStr">
+        <is>
+          <t>完全遮光・接触冷感UVハット</t>
+        </is>
+      </c>
+      <c r="B23" s="14" t="n">
+        <v>11960</v>
+      </c>
+      <c r="C23" s="14" t="n">
+        <v>2822</v>
+      </c>
+      <c r="D23" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="E23" s="14" t="n">
+        <v>9138</v>
+      </c>
+      <c r="F23" s="15" t="n">
+        <v>0.764</v>
+      </c>
+      <c r="G23" s="15" t="n">
+        <v>0.236</v>
+      </c>
+      <c r="H23" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="I23" s="13" t="inlineStr">
         <is>
           <t>−</t>
         </is>
       </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="11" t="inlineStr">
-        <is>
-          <t>完全遮光・接触冷感UVハット</t>
-        </is>
-      </c>
-      <c r="B23" s="12" t="n">
-        <v>11960</v>
-      </c>
-      <c r="C23" s="12" t="n">
-        <v>2822</v>
-      </c>
-      <c r="D23" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="E23" s="12" t="n">
-        <v>9138</v>
-      </c>
-      <c r="F23" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="G23" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="H23" s="11" t="inlineStr"/>
-      <c r="I23" s="12" t="n">
+      <c r="J23" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="K23" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="L23" s="13" t="inlineStr"/>
+      <c r="M23" s="14" t="n">
         <v>4569</v>
       </c>
-      <c r="J23" s="12" t="n">
+      <c r="N23" s="14" t="n">
         <v>41121</v>
       </c>
-      <c r="K23" s="11" t="inlineStr"/>
-      <c r="L23" s="11" t="inlineStr"/>
-      <c r="M23" s="11" t="inlineStr"/>
-      <c r="N23" s="11" t="inlineStr"/>
-      <c r="O23" s="11" t="inlineStr"/>
-      <c r="P23" s="11" t="inlineStr">
+      <c r="O23" s="13" t="inlineStr"/>
+      <c r="P23" s="13" t="inlineStr"/>
+      <c r="Q23" s="13" t="inlineStr"/>
+      <c r="R23" s="13" t="inlineStr"/>
+      <c r="S23" s="13" t="inlineStr"/>
+      <c r="T23" s="13" t="inlineStr">
         <is>
           <t>📦広告なし</t>
         </is>
       </c>
-      <c r="Q23" s="11" t="inlineStr">
-        <is>
-          <t>−</t>
+      <c r="U23" s="17" t="inlineStr">
+        <is>
+          <t>①広告ゼロで利益率76.4%。原価率23.6%は良好②日販ほぼゼロ。日傘・パーカーとのセット販売でクロスセルする方が費用対効果が高い③単独出稿は原価率が良いので秋の帽子需要期（10月）にテスト枠の候補</t>
         </is>
       </c>
     </row>
@@ -2365,79 +2714,107 @@
       <c r="E24" s="5" t="n">
         <v>6946</v>
       </c>
-      <c r="F24" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="G24" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="H24" s="4" t="inlineStr"/>
-      <c r="I24" s="5" t="n">
-        <v>0</v>
+      <c r="F24" s="6" t="n">
+        <v>0.696</v>
+      </c>
+      <c r="G24" s="6" t="n">
+        <v>0.304</v>
+      </c>
+      <c r="H24" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I24" s="4" t="inlineStr">
+        <is>
+          <t>−</t>
+        </is>
       </c>
       <c r="J24" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="K24" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="L24" s="4" t="inlineStr"/>
+      <c r="M24" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="N24" s="5" t="n">
         <v>6946</v>
       </c>
-      <c r="K24" s="4" t="inlineStr"/>
-      <c r="L24" s="4" t="inlineStr"/>
-      <c r="M24" s="4" t="inlineStr"/>
-      <c r="N24" s="4" t="inlineStr"/>
       <c r="O24" s="4" t="inlineStr"/>
-      <c r="P24" s="4" t="inlineStr">
+      <c r="P24" s="4" t="inlineStr"/>
+      <c r="Q24" s="4" t="inlineStr"/>
+      <c r="R24" s="4" t="inlineStr"/>
+      <c r="S24" s="4" t="inlineStr"/>
+      <c r="T24" s="4" t="inlineStr">
         <is>
           <t>📦広告なし</t>
         </is>
       </c>
-      <c r="Q24" s="4" t="inlineStr">
+      <c r="U24" s="12" t="inlineStr">
+        <is>
+          <t>①広告ゼロ・30日で1個。売価9,980円・原価3,034円で原価率30.4%は良好②秋冬需要（肩こり・ギフト）商品。11月のテスト枠候補として保留③今は何もしない</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="13" t="inlineStr">
+        <is>
+          <t>リカバリーサンダル</t>
+        </is>
+      </c>
+      <c r="B25" s="14" t="n">
+        <v>7960</v>
+      </c>
+      <c r="C25" s="14" t="n">
+        <v>2618</v>
+      </c>
+      <c r="D25" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="E25" s="14" t="n">
+        <v>5342</v>
+      </c>
+      <c r="F25" s="15" t="n">
+        <v>0.6711</v>
+      </c>
+      <c r="G25" s="15" t="n">
+        <v>0.3289</v>
+      </c>
+      <c r="H25" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="I25" s="13" t="inlineStr">
         <is>
           <t>−</t>
         </is>
       </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="11" t="inlineStr">
-        <is>
-          <t>リカバリーサンダル</t>
-        </is>
-      </c>
-      <c r="B25" s="12" t="n">
-        <v>7960</v>
-      </c>
-      <c r="C25" s="12" t="n">
-        <v>2618</v>
-      </c>
-      <c r="D25" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="E25" s="12" t="n">
-        <v>5342</v>
-      </c>
-      <c r="F25" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="G25" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="H25" s="11" t="inlineStr"/>
-      <c r="I25" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="J25" s="12" t="n">
+      <c r="J25" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="K25" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="L25" s="13" t="inlineStr"/>
+      <c r="M25" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="N25" s="14" t="n">
         <v>18697</v>
       </c>
-      <c r="K25" s="11" t="inlineStr"/>
-      <c r="L25" s="11" t="inlineStr"/>
-      <c r="M25" s="11" t="inlineStr"/>
-      <c r="N25" s="11" t="inlineStr"/>
-      <c r="O25" s="11" t="inlineStr"/>
-      <c r="P25" s="11" t="inlineStr">
+      <c r="O25" s="13" t="inlineStr"/>
+      <c r="P25" s="13" t="inlineStr"/>
+      <c r="Q25" s="13" t="inlineStr"/>
+      <c r="R25" s="13" t="inlineStr"/>
+      <c r="S25" s="13" t="inlineStr"/>
+      <c r="T25" s="13" t="inlineStr">
         <is>
           <t>📦広告なし</t>
         </is>
       </c>
-      <c r="Q25" s="11" t="inlineStr">
-        <is>
-          <t>−</t>
+      <c r="U25" s="17" t="inlineStr">
+        <is>
+          <t>①広告ゼロ・30日7個。原価率32.9%②サンダルは8月で需要終了。今から広告を出す価値はない③来春（4月）のテスト枠候補</t>
         </is>
       </c>
     </row>
@@ -2459,79 +2836,95 @@
       <c r="E26" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="F26" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="G26" s="5" t="n">
-        <v>0</v>
-      </c>
+      <c r="F26" s="4" t="inlineStr"/>
+      <c r="G26" s="4" t="inlineStr"/>
       <c r="H26" s="4" t="inlineStr"/>
-      <c r="I26" s="5" t="n">
-        <v>0</v>
+      <c r="I26" s="4" t="inlineStr">
+        <is>
+          <t>−</t>
+        </is>
       </c>
       <c r="J26" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="K26" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="L26" s="4" t="inlineStr"/>
+      <c r="M26" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="N26" s="5" t="n">
         <v>56700</v>
       </c>
-      <c r="K26" s="4" t="inlineStr"/>
-      <c r="L26" s="4" t="inlineStr"/>
-      <c r="M26" s="4" t="inlineStr"/>
-      <c r="N26" s="4" t="inlineStr"/>
       <c r="O26" s="4" t="inlineStr"/>
-      <c r="P26" s="4" t="inlineStr">
+      <c r="P26" s="4" t="inlineStr"/>
+      <c r="Q26" s="4" t="inlineStr"/>
+      <c r="R26" s="4" t="inlineStr"/>
+      <c r="S26" s="4" t="inlineStr"/>
+      <c r="T26" s="4" t="inlineStr">
         <is>
           <t>📦広告なし</t>
         </is>
       </c>
-      <c r="Q26" s="4" t="inlineStr">
+      <c r="U26" s="12" t="inlineStr">
+        <is>
+          <t>①30日売上8.4万円・広告ゼロ。原価率32.3%②シャワーヘッドは秋冬に需要が上がる（入浴時間の増加）③9月のテスト枠の第一候補。原価2,255円・売価6,980円で分岐MER1.48は良好</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="13" t="inlineStr">
+        <is>
+          <t>姿勢サポートベルト</t>
+        </is>
+      </c>
+      <c r="B27" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="C27" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="D27" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="E27" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="F27" s="13" t="inlineStr"/>
+      <c r="G27" s="13" t="inlineStr"/>
+      <c r="H27" s="13" t="inlineStr"/>
+      <c r="I27" s="13" t="inlineStr">
         <is>
           <t>−</t>
         </is>
       </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="11" t="inlineStr">
-        <is>
-          <t>姿勢サポートベルト</t>
-        </is>
-      </c>
-      <c r="B27" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="C27" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="D27" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="E27" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="F27" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="G27" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="H27" s="11" t="inlineStr"/>
-      <c r="I27" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="J27" s="12" t="n">
+      <c r="J27" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="K27" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="L27" s="13" t="inlineStr"/>
+      <c r="M27" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="N27" s="14" t="n">
         <v>4551</v>
       </c>
-      <c r="K27" s="11" t="inlineStr"/>
-      <c r="L27" s="11" t="inlineStr"/>
-      <c r="M27" s="11" t="inlineStr"/>
-      <c r="N27" s="11" t="inlineStr"/>
-      <c r="O27" s="11" t="inlineStr"/>
-      <c r="P27" s="11" t="inlineStr">
+      <c r="O27" s="13" t="inlineStr"/>
+      <c r="P27" s="13" t="inlineStr"/>
+      <c r="Q27" s="13" t="inlineStr"/>
+      <c r="R27" s="13" t="inlineStr"/>
+      <c r="S27" s="13" t="inlineStr"/>
+      <c r="T27" s="13" t="inlineStr">
         <is>
           <t>📦広告なし</t>
         </is>
       </c>
-      <c r="Q27" s="11" t="inlineStr">
-        <is>
-          <t>−</t>
+      <c r="U27" s="17" t="inlineStr">
+        <is>
+          <t>①30日1個。原価率24.1%は良好だが需要が立っていない②在庫リスクなし。放置で問題なし</t>
         </is>
       </c>
     </row>
@@ -2553,32 +2946,40 @@
       <c r="E28" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="F28" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="G28" s="5" t="n">
-        <v>0</v>
-      </c>
+      <c r="F28" s="4" t="inlineStr"/>
+      <c r="G28" s="4" t="inlineStr"/>
       <c r="H28" s="4" t="inlineStr"/>
-      <c r="I28" s="5" t="n">
-        <v>0</v>
+      <c r="I28" s="4" t="inlineStr">
+        <is>
+          <t>−</t>
+        </is>
       </c>
       <c r="J28" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="K28" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="L28" s="4" t="inlineStr"/>
+      <c r="M28" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="N28" s="5" t="n">
         <v>4332</v>
       </c>
-      <c r="K28" s="4" t="inlineStr"/>
-      <c r="L28" s="4" t="inlineStr"/>
-      <c r="M28" s="4" t="inlineStr"/>
-      <c r="N28" s="4" t="inlineStr"/>
       <c r="O28" s="4" t="inlineStr"/>
-      <c r="P28" s="4" t="inlineStr">
+      <c r="P28" s="4" t="inlineStr"/>
+      <c r="Q28" s="4" t="inlineStr"/>
+      <c r="R28" s="4" t="inlineStr"/>
+      <c r="S28" s="4" t="inlineStr"/>
+      <c r="T28" s="4" t="inlineStr">
         <is>
           <t>📦広告なし</t>
         </is>
       </c>
-      <c r="Q28" s="4" t="inlineStr">
-        <is>
-          <t>−</t>
+      <c r="U28" s="12" t="inlineStr">
+        <is>
+          <t>①30日1個。7/25改定で原価1,910→1,648円（−262円）と最大の値下げ幅②原価率27.6%まで改善。売価5,980円で分岐MER1.38③秋冬の「おうち時間」需要でテスト枠候補</t>
         </is>
       </c>
     </row>

</xml_diff>